<commit_message>
Nueva versión: Bugs criticos corregidos pero avg GAP del 63%
</commit_message>
<xml_diff>
--- a/DRL_Routing_Summary_stochastic_sigma10%_AM.xlsx
+++ b/DRL_Routing_Summary_stochastic_sigma10%_AM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a9faf7a5fe1343c6/Desktop/Maestria/Tesis MSc/RoutingModel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="11_8B418FE7A3AC9DB39A77A79623358AD3C21CA036" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A43F6FB-DFA8-45E3-BF80-140DABD45E9B}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="11_8B418FE7CD8C9DC923EC111537358AD3C21C5585" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA0D36EC-DEB9-4020-84F1-533CC9A82636}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="88">
   <si>
     <t>Start Node</t>
   </si>
@@ -45,7 +45,7 @@
     <t>DRL Route</t>
   </si>
   <si>
-    <t>DRL Reward</t>
+    <t>DRL Det Reward</t>
   </si>
   <si>
     <t>DRL Duration</t>
@@ -108,6 +108,21 @@
     <t>GA Route</t>
   </si>
   <si>
+    <t>GA Reward</t>
+  </si>
+  <si>
+    <t>GA Duration</t>
+  </si>
+  <si>
+    <t>GA Valid</t>
+  </si>
+  <si>
+    <t>LNS Status</t>
+  </si>
+  <si>
+    <t>LNS Route</t>
+  </si>
+  <si>
     <t>LNS Reward</t>
   </si>
   <si>
@@ -117,6 +132,21 @@
     <t>LNS Valid</t>
   </si>
   <si>
+    <t>HGA-LNS Status</t>
+  </si>
+  <si>
+    <t>HGA-LNS Route</t>
+  </si>
+  <si>
+    <t>HGA-LNS Reward</t>
+  </si>
+  <si>
+    <t>HGA-LNS Duration</t>
+  </si>
+  <si>
+    <t>HGA-LNS Valid</t>
+  </si>
+  <si>
     <t>DRL Gap (%)</t>
   </si>
   <si>
@@ -129,112 +159,109 @@
     <t>LNS Gap (%)</t>
   </si>
   <si>
-    <t>[0, 6, 2, 1, 0]</t>
+    <t>[0, 7, 6, 0]</t>
   </si>
   <si>
     <t>Optimal</t>
   </si>
   <si>
-    <t>[0, 6, 1, 2, 0]</t>
+    <t>[0, 6, 1, 7, 0]</t>
   </si>
   <si>
     <t>[0, 2, 1, 6, 0]</t>
   </si>
   <si>
-    <t>[0, 1, 2, 6, 0]</t>
+    <t>[1, 0, 6, 1]</t>
+  </si>
+  <si>
+    <t>[1, 6, 0, 8, 1]</t>
   </si>
   <si>
     <t>[1, 4, 1]</t>
   </si>
   <si>
-    <t>[1, 7, 2, 6, 1]</t>
-  </si>
-  <si>
-    <t>[1, 5, 9, 1]</t>
-  </si>
-  <si>
-    <t>[1, 0, 2, 6, 1]</t>
-  </si>
-  <si>
-    <t>[2, 0, 7, 2]</t>
-  </si>
-  <si>
-    <t>[2, 8, 0, 7, 2]</t>
-  </si>
-  <si>
-    <t>[2, 5, 3, 4, 2]</t>
-  </si>
-  <si>
-    <t>[2, 1, 4, 2]</t>
-  </si>
-  <si>
-    <t>[3, 5, 2, 3]</t>
-  </si>
-  <si>
-    <t>[3, 4, 2, 5, 3]</t>
-  </si>
-  <si>
-    <t>[3, 4, 5, 9, 3]</t>
-  </si>
-  <si>
-    <t>[3, 4, 9, 5, 3]</t>
-  </si>
-  <si>
-    <t>[4, 2, 8, 1, 4]</t>
-  </si>
-  <si>
-    <t>[4, 1, 8, 2, 4]</t>
+    <t>[1, 6, 0, 7, 1]</t>
+  </si>
+  <si>
+    <t>[2, 7, 0, 2]</t>
+  </si>
+  <si>
+    <t>[2, 8, 1, 7, 2]</t>
+  </si>
+  <si>
+    <t>[2, 5, 2]</t>
+  </si>
+  <si>
+    <t>[2, 8, 1, 6, 2]</t>
+  </si>
+  <si>
+    <t>[3, 5, 3]</t>
+  </si>
+  <si>
+    <t>[3, 4, 5, 3]</t>
+  </si>
+  <si>
+    <t>[4, 2, 3, 4]</t>
   </si>
   <si>
     <t>[4, 1, 2, 4]</t>
   </si>
   <si>
-    <t>[5, 2, 3, 5]</t>
-  </si>
-  <si>
-    <t>[5, 1, 5]</t>
-  </si>
-  <si>
-    <t>[5, 1, 9, 5]</t>
-  </si>
-  <si>
-    <t>[5, 3, 4, 2, 5]</t>
-  </si>
-  <si>
-    <t>[6, 2, 7, 6]</t>
-  </si>
-  <si>
-    <t>[6, 0, 2, 7, 6]</t>
-  </si>
-  <si>
-    <t>[6, 2, 7, 1, 6]</t>
-  </si>
-  <si>
-    <t>[7, 0, 6, 1, 7]</t>
-  </si>
-  <si>
-    <t>[7, 2, 9, 1, 7]</t>
-  </si>
-  <si>
-    <t>[8, 7, 0, 6, 8]</t>
-  </si>
-  <si>
-    <t>[8, 6, 1, 2, 8]</t>
-  </si>
-  <si>
-    <t>[8, 5, 8]</t>
-  </si>
-  <si>
-    <t>[9, 6, 0, 1, 9]</t>
-  </si>
-  <si>
-    <t>[9, 2, 1, 6, 9]</t>
+    <t>[5, 2, 5]</t>
+  </si>
+  <si>
+    <t>[6, 7, 6]</t>
+  </si>
+  <si>
+    <t>[6, 7, 2, 8, 6]</t>
+  </si>
+  <si>
+    <t>[6, 2, 8, 1, 6]</t>
+  </si>
+  <si>
+    <t>[6, 2, 1, 8, 6]</t>
+  </si>
+  <si>
+    <t>[7, 6, 7]</t>
+  </si>
+  <si>
+    <t>[7, 2, 8, 1, 7]</t>
+  </si>
+  <si>
+    <t>[8, 0, 7, 8]</t>
+  </si>
+  <si>
+    <t>[8, 1, 6, 0, 8]</t>
+  </si>
+  <si>
+    <t>[8, 1, 2, 8]</t>
+  </si>
+  <si>
+    <t>[8, 1, 0, 2, 8]</t>
+  </si>
+  <si>
+    <t>[8, 2, 1, 0, 8]</t>
   </si>
   <si>
     <t>[9, 2, 5, 9]</t>
   </si>
   <si>
-    <t>[9, 2, 7, 6, 9]</t>
+    <t>[9, 2, 6, 1, 9]</t>
+  </si>
+  <si>
+    <t>[9]</t>
+  </si>
+  <si>
+    <t>-inf</t>
+  </si>
+  <si>
+    <t>Infeasible</t>
+  </si>
+  <si>
+    <t>inf</t>
+  </si>
+  <si>
+    <t>[9, 1, 0, 2, 9]</t>
   </si>
   <si>
     <t>Model</t>
@@ -256,6 +283,12 @@
   </si>
   <si>
     <t>GA Avg</t>
+  </si>
+  <si>
+    <t>LNS Avg</t>
+  </si>
+  <si>
+    <t>HGA-LNS Avg</t>
   </si>
   <si>
     <t>DRL Training Time</t>
@@ -627,37 +660,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AE13"/>
+  <dimension ref="A1:AP11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="11.109375" customWidth="1"/>
-    <col min="5" max="5" width="11.88671875" customWidth="1"/>
-    <col min="6" max="6" width="11.5546875" customWidth="1"/>
-    <col min="7" max="7" width="17.77734375" customWidth="1"/>
-    <col min="8" max="8" width="13.6640625" customWidth="1"/>
-    <col min="9" max="9" width="8.88671875" customWidth="1"/>
-    <col min="10" max="10" width="12.109375" customWidth="1"/>
-    <col min="11" max="11" width="15.77734375" customWidth="1"/>
+    <col min="4" max="4" width="15.109375" customWidth="1"/>
     <col min="12" max="12" width="14.44140625" customWidth="1"/>
-    <col min="13" max="13" width="15.88671875" customWidth="1"/>
-    <col min="14" max="15" width="14.5546875" customWidth="1"/>
-    <col min="16" max="16" width="14.77734375" customWidth="1"/>
-    <col min="17" max="17" width="16" customWidth="1"/>
-    <col min="18" max="18" width="14.21875" customWidth="1"/>
-    <col min="19" max="19" width="13.21875" customWidth="1"/>
-    <col min="20" max="20" width="14.109375" customWidth="1"/>
-    <col min="21" max="21" width="13.21875" customWidth="1"/>
-    <col min="22" max="22" width="15" customWidth="1"/>
-    <col min="25" max="25" width="16.21875" customWidth="1"/>
-    <col min="27" max="27" width="15.33203125" customWidth="1"/>
-    <col min="28" max="28" width="15.21875" customWidth="1"/>
-    <col min="29" max="29" width="15.5546875" customWidth="1"/>
-    <col min="30" max="30" width="17.44140625" customWidth="1"/>
-    <col min="31" max="31" width="16.6640625" customWidth="1"/>
+    <col min="16" max="16" width="17.33203125" customWidth="1"/>
+    <col min="20" max="20" width="14.6640625" customWidth="1"/>
+    <col min="25" max="25" width="16.33203125" customWidth="1"/>
+    <col min="30" max="30" width="14.33203125" customWidth="1"/>
+    <col min="33" max="33" width="15" customWidth="1"/>
+    <col min="34" max="34" width="19.109375" customWidth="1"/>
+    <col min="35" max="35" width="16.88671875" customWidth="1"/>
+    <col min="36" max="36" width="13.6640625" customWidth="1"/>
+    <col min="40" max="40" width="13.77734375" customWidth="1"/>
+    <col min="41" max="41" width="14.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -751,973 +771,1309 @@
       <c r="AE1" s="1" t="s">
         <v>30</v>
       </c>
+      <c r="AF1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AL1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AM1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AO1" s="1" t="s">
+        <v>40</v>
+      </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>0</v>
       </c>
       <c r="B2">
-        <v>47</v>
+        <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="D2">
-        <v>4403</v>
+        <v>2314</v>
       </c>
       <c r="E2">
-        <v>56.8</v>
+        <v>46.06</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
       </c>
       <c r="G2">
-        <v>4355.0707028250999</v>
+        <v>2335.3456633935248</v>
       </c>
       <c r="H2">
-        <v>444.22876624471252</v>
+        <v>294.92221592010389</v>
       </c>
       <c r="I2">
         <v>100</v>
       </c>
       <c r="J2" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="K2" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="L2">
-        <v>4973</v>
+        <v>3921</v>
       </c>
       <c r="M2">
-        <v>66.2</v>
+        <v>74.17</v>
       </c>
       <c r="N2" t="b">
         <v>1</v>
       </c>
       <c r="O2" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="P2">
-        <v>3960</v>
+        <v>3306</v>
       </c>
       <c r="Q2">
-        <v>65.599999999999994</v>
+        <v>72.849999999999994</v>
       </c>
       <c r="R2" t="b">
         <v>1</v>
       </c>
       <c r="S2" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="T2">
-        <v>4403</v>
+        <v>3306</v>
       </c>
       <c r="U2">
-        <v>56.8</v>
+        <v>72.849999999999994</v>
       </c>
       <c r="V2" t="b">
         <v>1</v>
       </c>
       <c r="W2" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="X2" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="Y2">
-        <v>4973</v>
+        <v>3921</v>
       </c>
       <c r="Z2">
-        <v>66.2</v>
+        <v>74.17</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
       </c>
-      <c r="AB2">
-        <v>11.46189422883571</v>
-      </c>
-      <c r="AC2">
-        <v>20.369997989141361</v>
+      <c r="AB2" t="s">
+        <v>42</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>44</v>
       </c>
       <c r="AD2">
-        <v>11.46189422883571</v>
+        <v>3306</v>
       </c>
       <c r="AE2">
+        <v>72.849999999999994</v>
+      </c>
+      <c r="AF2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH2" t="s">
+        <v>43</v>
+      </c>
+      <c r="AI2">
+        <v>3921</v>
+      </c>
+      <c r="AJ2">
+        <v>74.17</v>
+      </c>
+      <c r="AK2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL2">
+        <v>40.984442744197906</v>
+      </c>
+      <c r="AM2">
+        <v>15.68477429227238</v>
+      </c>
+      <c r="AN2">
+        <v>15.68477429227238</v>
+      </c>
+      <c r="AO2">
+        <v>15.68477429227238</v>
+      </c>
+      <c r="AP2">
+        <f>1-AI2/L2</f>
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="D3">
-        <v>4724</v>
+        <v>2055</v>
       </c>
       <c r="E3">
-        <v>65.900000000000006</v>
+        <v>41.34</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
       </c>
       <c r="G3">
-        <v>4680.5560755790266</v>
+        <v>2156.3053470928312</v>
       </c>
       <c r="H3">
-        <v>296.95403369319951</v>
+        <v>342.54715715840217</v>
       </c>
       <c r="I3">
         <v>100</v>
       </c>
       <c r="J3" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="K3" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="L3">
-        <v>5153</v>
+        <v>3338</v>
       </c>
       <c r="M3">
-        <v>74.399999999999991</v>
+        <v>67.180000000000007</v>
       </c>
       <c r="N3" t="b">
         <v>1</v>
       </c>
       <c r="O3" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="P3">
-        <v>-1995</v>
+        <v>2765</v>
       </c>
       <c r="Q3">
-        <v>75</v>
+        <v>73.19</v>
       </c>
       <c r="R3" t="b">
         <v>1</v>
       </c>
       <c r="S3" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="T3">
-        <v>-1995</v>
+        <v>2765</v>
       </c>
       <c r="U3">
-        <v>75</v>
+        <v>73.19</v>
       </c>
       <c r="V3" t="b">
         <v>1</v>
       </c>
       <c r="W3" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="X3" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="Y3">
-        <v>4794</v>
+        <v>3298</v>
       </c>
       <c r="Z3">
-        <v>66.2</v>
+        <v>74.169999999999987</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
       </c>
-      <c r="AB3">
-        <v>8.3252474286823208</v>
-      </c>
-      <c r="AC3">
-        <v>138.71531146904721</v>
+      <c r="AB3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>47</v>
       </c>
       <c r="AD3">
-        <v>138.71531146904721</v>
+        <v>2765</v>
       </c>
       <c r="AE3">
-        <v>6.9668154473122446</v>
+        <v>73.19</v>
+      </c>
+      <c r="AF3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH3" t="s">
+        <v>46</v>
+      </c>
+      <c r="AI3">
+        <v>3338</v>
+      </c>
+      <c r="AJ3">
+        <v>67.180000000000007</v>
+      </c>
+      <c r="AK3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL3">
+        <v>38.4361893349311</v>
+      </c>
+      <c r="AM3">
+        <v>17.165967645296579</v>
+      </c>
+      <c r="AN3">
+        <v>17.165967645296579</v>
+      </c>
+      <c r="AO3">
+        <v>17.165967645296579</v>
+      </c>
+      <c r="AP3">
+        <f t="shared" ref="AP3:AP11" si="0">1-AI3/L3</f>
+        <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="C4" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="D4">
-        <v>3213</v>
+        <v>2317</v>
       </c>
       <c r="E4">
-        <v>68.3</v>
+        <v>76.42</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
       </c>
       <c r="G4">
-        <v>3235.7185708012248</v>
+        <v>2336.547064110503</v>
       </c>
       <c r="H4">
-        <v>335.64455756205439</v>
+        <v>313.6742568385032</v>
       </c>
       <c r="I4">
         <v>100</v>
       </c>
       <c r="J4" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="K4" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="L4">
-        <v>3968</v>
+        <v>3527</v>
       </c>
       <c r="M4">
-        <v>71.5</v>
+        <v>70.02</v>
       </c>
       <c r="N4" t="b">
         <v>1</v>
       </c>
       <c r="O4" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="P4">
-        <v>3508</v>
+        <v>2635</v>
       </c>
       <c r="Q4">
-        <v>76.3</v>
+        <v>73.8</v>
       </c>
       <c r="R4" t="b">
         <v>1</v>
       </c>
       <c r="S4" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="T4">
-        <v>3508</v>
+        <v>2635</v>
       </c>
       <c r="U4">
-        <v>76.3</v>
+        <v>73.8</v>
       </c>
       <c r="V4" t="b">
         <v>1</v>
       </c>
       <c r="W4" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="X4" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="Y4">
-        <v>3906</v>
+        <v>3046</v>
       </c>
       <c r="Z4">
-        <v>69.599999999999994</v>
+        <v>55.1</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
       </c>
-      <c r="AB4">
-        <v>19.02721774193548</v>
-      </c>
-      <c r="AC4">
-        <v>11.59274193548387</v>
+      <c r="AB4" t="s">
+        <v>42</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>51</v>
       </c>
       <c r="AD4">
-        <v>11.59274193548387</v>
+        <v>2635</v>
       </c>
       <c r="AE4">
-        <v>1.5625</v>
+        <v>73.8</v>
+      </c>
+      <c r="AF4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG4" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH4" t="s">
+        <v>50</v>
+      </c>
+      <c r="AI4">
+        <v>3527</v>
+      </c>
+      <c r="AJ4">
+        <v>70.02000000000001</v>
+      </c>
+      <c r="AK4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL4">
+        <v>34.306776297136373</v>
+      </c>
+      <c r="AM4">
+        <v>25.29061525375673</v>
+      </c>
+      <c r="AN4">
+        <v>25.29061525375673</v>
+      </c>
+      <c r="AO4">
+        <v>25.29061525375673</v>
+      </c>
+      <c r="AP4">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="C5" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="D5">
-        <v>2855</v>
+        <v>1109</v>
       </c>
       <c r="E5">
-        <v>74.900000000000006</v>
+        <v>26.24</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>2805.0235672575059</v>
+        <v>1133.903036548925</v>
       </c>
       <c r="H5">
-        <v>356.30566752315428</v>
+        <v>271.25861740600612</v>
       </c>
       <c r="I5">
         <v>100</v>
       </c>
       <c r="J5" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="K5" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="L5">
-        <v>3733</v>
+        <v>1777</v>
       </c>
       <c r="M5">
-        <v>76.3</v>
+        <v>42.15</v>
       </c>
       <c r="N5" t="b">
         <v>1</v>
       </c>
       <c r="O5" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="P5">
-        <v>-4144</v>
+        <v>1777</v>
       </c>
       <c r="Q5">
-        <v>72.599999999999994</v>
+        <v>42.15</v>
       </c>
       <c r="R5" t="b">
         <v>1</v>
       </c>
       <c r="S5" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="T5">
-        <v>-3263</v>
+        <v>1777</v>
       </c>
       <c r="U5">
-        <v>62.8</v>
+        <v>42.15</v>
       </c>
       <c r="V5" t="b">
         <v>1</v>
       </c>
       <c r="W5" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="X5" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="Y5">
-        <v>3733</v>
+        <v>1777</v>
       </c>
       <c r="Z5">
-        <v>76.3</v>
+        <v>42.15</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
       </c>
-      <c r="AB5">
-        <v>23.519957139030272</v>
-      </c>
-      <c r="AC5">
-        <v>211.00991159924999</v>
+      <c r="AB5" t="s">
+        <v>42</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>54</v>
       </c>
       <c r="AD5">
-        <v>187.40959014197699</v>
+        <v>1777</v>
       </c>
       <c r="AE5">
+        <v>42.15</v>
+      </c>
+      <c r="AF5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG5" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH5" t="s">
+        <v>54</v>
+      </c>
+      <c r="AI5">
+        <v>1777</v>
+      </c>
+      <c r="AJ5">
+        <v>42.15</v>
+      </c>
+      <c r="AK5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL5">
+        <v>37.591446257737758</v>
+      </c>
+      <c r="AM5">
+        <v>0</v>
+      </c>
+      <c r="AN5">
+        <v>0</v>
+      </c>
+      <c r="AO5">
+        <v>0</v>
+      </c>
+      <c r="AP5">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>4</v>
       </c>
       <c r="B6">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C6" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="D6">
-        <v>4961</v>
+        <v>2664</v>
       </c>
       <c r="E6">
-        <v>73</v>
+        <v>68.070000000000007</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
       </c>
       <c r="G6">
-        <v>5016.5030352488911</v>
+        <v>2698.5698819653289</v>
       </c>
       <c r="H6">
-        <v>336.21459581352519</v>
+        <v>402.03498569843828</v>
       </c>
       <c r="I6">
         <v>100</v>
       </c>
       <c r="J6" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="K6" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="L6">
-        <v>4961</v>
+        <v>5508</v>
       </c>
       <c r="M6">
-        <v>73</v>
+        <v>76.709999999999994</v>
       </c>
       <c r="N6" t="b">
         <v>1</v>
       </c>
       <c r="O6" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="P6">
-        <v>4814</v>
+        <v>5508</v>
       </c>
       <c r="Q6">
-        <v>69.099999999999994</v>
+        <v>76.709999999999994</v>
       </c>
       <c r="R6" t="b">
         <v>1</v>
       </c>
       <c r="S6" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="T6">
-        <v>4814</v>
+        <v>5508</v>
       </c>
       <c r="U6">
-        <v>69.099999999999994</v>
+        <v>76.709999999999994</v>
       </c>
       <c r="V6" t="b">
         <v>1</v>
       </c>
       <c r="W6" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="X6" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="Y6">
-        <v>4961</v>
+        <v>5508</v>
       </c>
       <c r="Z6">
-        <v>73</v>
+        <v>76.709999999999994</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
       </c>
-      <c r="AB6">
-        <v>0</v>
-      </c>
-      <c r="AC6">
-        <v>2.963112275750857</v>
+      <c r="AB6" t="s">
+        <v>42</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>56</v>
       </c>
       <c r="AD6">
-        <v>2.963112275750857</v>
+        <v>5508</v>
       </c>
       <c r="AE6">
+        <v>76.709999999999994</v>
+      </c>
+      <c r="AF6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG6" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AI6">
+        <v>5508</v>
+      </c>
+      <c r="AJ6">
+        <v>76.709999999999994</v>
+      </c>
+      <c r="AK6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL6">
+        <v>51.633986928104576</v>
+      </c>
+      <c r="AM6">
+        <v>0</v>
+      </c>
+      <c r="AN6">
+        <v>0</v>
+      </c>
+      <c r="AO6">
+        <v>0</v>
+      </c>
+      <c r="AP6">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>5</v>
       </c>
       <c r="B7">
-        <v>66</v>
+        <v>83</v>
       </c>
       <c r="C7" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D7">
-        <v>3416</v>
+        <v>2959</v>
       </c>
       <c r="E7">
-        <v>74.900000000000006</v>
+        <v>73.8</v>
       </c>
       <c r="F7" t="b">
         <v>1</v>
       </c>
       <c r="G7">
-        <v>3432.4471536167011</v>
+        <v>2947.9149097342638</v>
       </c>
       <c r="H7">
-        <v>363.92415914948867</v>
+        <v>328.03726995268232</v>
       </c>
       <c r="I7">
         <v>100</v>
       </c>
       <c r="J7" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="K7" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="L7">
-        <v>4831</v>
+        <v>2959</v>
       </c>
       <c r="M7">
-        <v>74.8</v>
+        <v>73.8</v>
       </c>
       <c r="N7" t="b">
         <v>1</v>
       </c>
       <c r="O7" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="P7">
-        <v>-1602</v>
+        <v>2959</v>
       </c>
       <c r="Q7">
-        <v>74.900000000000006</v>
+        <v>73.8</v>
       </c>
       <c r="R7" t="b">
         <v>1</v>
       </c>
       <c r="S7" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="T7">
-        <v>-1602</v>
+        <v>2959</v>
       </c>
       <c r="U7">
-        <v>74.900000000000006</v>
+        <v>73.8</v>
       </c>
       <c r="V7" t="b">
         <v>1</v>
       </c>
       <c r="W7" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="X7" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="Y7">
-        <v>3490</v>
+        <v>2959</v>
       </c>
       <c r="Z7">
-        <v>76.300000000000011</v>
+        <v>73.8</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
       </c>
-      <c r="AB7">
-        <v>29.29000206996481</v>
-      </c>
-      <c r="AC7">
-        <v>133.1608362657835</v>
+      <c r="AB7" t="s">
+        <v>42</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>57</v>
       </c>
       <c r="AD7">
-        <v>133.1608362657835</v>
+        <v>2959</v>
       </c>
       <c r="AE7">
-        <v>27.758228110122129</v>
+        <v>73.8</v>
+      </c>
+      <c r="AF7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG7" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH7" t="s">
+        <v>57</v>
+      </c>
+      <c r="AI7">
+        <v>2959</v>
+      </c>
+      <c r="AJ7">
+        <v>73.8</v>
+      </c>
+      <c r="AK7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL7">
+        <v>0</v>
+      </c>
+      <c r="AM7">
+        <v>0</v>
+      </c>
+      <c r="AN7">
+        <v>0</v>
+      </c>
+      <c r="AO7">
+        <v>0</v>
+      </c>
+      <c r="AP7">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>6</v>
       </c>
       <c r="B8">
-        <v>64</v>
+        <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D8">
-        <v>3719</v>
+        <v>872</v>
       </c>
       <c r="E8">
-        <v>49.099999999999987</v>
+        <v>17.260000000000002</v>
       </c>
       <c r="F8" t="b">
         <v>1</v>
       </c>
       <c r="G8">
-        <v>3661.754741472223</v>
+        <v>899.81989485242912</v>
       </c>
       <c r="H8">
-        <v>338.15327146932083</v>
+        <v>258.84282261065869</v>
       </c>
       <c r="I8">
         <v>100</v>
       </c>
       <c r="J8" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="K8" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="L8">
-        <v>4894</v>
+        <v>3552</v>
       </c>
       <c r="M8">
-        <v>69.3</v>
+        <v>54.48</v>
       </c>
       <c r="N8" t="b">
         <v>1</v>
       </c>
       <c r="O8" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="P8">
-        <v>4622</v>
+        <v>3005</v>
       </c>
       <c r="Q8">
-        <v>74.400000000000006</v>
+        <v>55.1</v>
       </c>
       <c r="R8" t="b">
         <v>1</v>
       </c>
       <c r="S8" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="T8">
-        <v>4622</v>
+        <v>3067</v>
       </c>
       <c r="U8">
-        <v>74.400000000000006</v>
+        <v>63.03</v>
       </c>
       <c r="V8" t="b">
         <v>1</v>
       </c>
       <c r="W8" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="X8" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="Y8">
-        <v>4894</v>
+        <v>3552</v>
       </c>
       <c r="Z8">
-        <v>69.3</v>
+        <v>54.48</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
       </c>
-      <c r="AB8">
-        <v>24.00899060073559</v>
-      </c>
-      <c r="AC8">
-        <v>5.5578259092766658</v>
+      <c r="AB8" t="s">
+        <v>42</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>60</v>
       </c>
       <c r="AD8">
-        <v>5.5578259092766658</v>
+        <v>3005</v>
       </c>
       <c r="AE8">
+        <v>55.1</v>
+      </c>
+      <c r="AF8" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG8" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH8" t="s">
+        <v>59</v>
+      </c>
+      <c r="AI8">
+        <v>3552</v>
+      </c>
+      <c r="AJ8">
+        <v>54.48</v>
+      </c>
+      <c r="AK8" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL8">
+        <v>75.450450450450447</v>
+      </c>
+      <c r="AM8">
+        <v>15.39977477477477</v>
+      </c>
+      <c r="AN8">
+        <v>13.65427927927928</v>
+      </c>
+      <c r="AO8">
+        <v>15.39977477477477</v>
+      </c>
+      <c r="AP8">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>7</v>
       </c>
       <c r="B9">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="C9" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="D9">
-        <v>3502</v>
+        <v>894</v>
       </c>
       <c r="E9">
-        <v>66.8</v>
+        <v>17.260000000000002</v>
       </c>
       <c r="F9" t="b">
         <v>1</v>
       </c>
       <c r="G9">
-        <v>3547.279159140428</v>
+        <v>857.88788365618939</v>
       </c>
       <c r="H9">
-        <v>387.70185657207128</v>
+        <v>282.68644545330102</v>
       </c>
       <c r="I9">
         <v>100</v>
       </c>
       <c r="J9" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="K9" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="L9">
-        <v>6128</v>
+        <v>3390</v>
       </c>
       <c r="M9">
-        <v>76.8</v>
+        <v>70.02</v>
       </c>
       <c r="N9" t="b">
         <v>1</v>
       </c>
       <c r="O9" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="P9">
-        <v>6128</v>
+        <v>3390</v>
       </c>
       <c r="Q9">
-        <v>76.8</v>
+        <v>70.02</v>
       </c>
       <c r="R9" t="b">
         <v>1</v>
       </c>
       <c r="S9" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="T9">
-        <v>6128</v>
+        <v>3390</v>
       </c>
       <c r="U9">
-        <v>76.8</v>
+        <v>70.02</v>
       </c>
       <c r="V9" t="b">
         <v>1</v>
       </c>
       <c r="W9" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="X9" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="Y9">
-        <v>6128</v>
+        <v>3390</v>
       </c>
       <c r="Z9">
-        <v>76.8</v>
+        <v>70.02</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
       </c>
-      <c r="AB9">
-        <v>42.85248041775457</v>
-      </c>
-      <c r="AC9">
-        <v>0</v>
+      <c r="AB9" t="s">
+        <v>42</v>
+      </c>
+      <c r="AC9" t="s">
+        <v>63</v>
       </c>
       <c r="AD9">
-        <v>0</v>
+        <v>3390</v>
       </c>
       <c r="AE9">
+        <v>70.02</v>
+      </c>
+      <c r="AF9" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG9" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH9" t="s">
+        <v>63</v>
+      </c>
+      <c r="AI9">
+        <v>3390</v>
+      </c>
+      <c r="AJ9">
+        <v>70.02</v>
+      </c>
+      <c r="AK9" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL9">
+        <v>73.628318584070797</v>
+      </c>
+      <c r="AM9">
+        <v>0</v>
+      </c>
+      <c r="AN9">
+        <v>0</v>
+      </c>
+      <c r="AO9">
+        <v>0</v>
+      </c>
+      <c r="AP9">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>8</v>
       </c>
       <c r="B10">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="C10" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="D10">
-        <v>3406</v>
+        <v>667</v>
       </c>
       <c r="E10">
-        <v>63.000000000000007</v>
+        <v>65.45</v>
       </c>
       <c r="F10" t="b">
         <v>1</v>
       </c>
       <c r="G10">
-        <v>3430.8570980299141</v>
+        <v>647.22446688879745</v>
       </c>
       <c r="H10">
-        <v>354.56198797382859</v>
+        <v>332.38245356187741</v>
       </c>
       <c r="I10">
         <v>100</v>
       </c>
       <c r="J10" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="K10" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="L10">
-        <v>3786</v>
+        <v>3338</v>
       </c>
       <c r="M10">
-        <v>45.4</v>
+        <v>67.180000000000007</v>
       </c>
       <c r="N10" t="b">
         <v>1</v>
       </c>
       <c r="O10" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="P10">
-        <v>3632</v>
+        <v>735</v>
       </c>
       <c r="Q10">
-        <v>76.8</v>
+        <v>37.81</v>
       </c>
       <c r="R10" t="b">
         <v>1</v>
       </c>
       <c r="S10" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="T10">
-        <v>3632</v>
+        <v>1255</v>
       </c>
       <c r="U10">
-        <v>76.8</v>
+        <v>60.95</v>
       </c>
       <c r="V10" t="b">
         <v>1</v>
       </c>
       <c r="W10" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="X10" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="Y10">
-        <v>3632</v>
+        <v>2612</v>
       </c>
       <c r="Z10">
-        <v>76.8</v>
+        <v>59.17</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
       </c>
-      <c r="AB10">
-        <v>10.03697834125726</v>
-      </c>
-      <c r="AC10">
-        <v>4.0676175382989959</v>
+      <c r="AB10" t="s">
+        <v>42</v>
+      </c>
+      <c r="AC10" t="s">
+        <v>66</v>
       </c>
       <c r="AD10">
-        <v>4.0676175382989959</v>
+        <v>735</v>
       </c>
       <c r="AE10">
-        <v>4.0676175382989959</v>
+        <v>37.81</v>
+      </c>
+      <c r="AF10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG10" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH10" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI10">
+        <v>3338</v>
+      </c>
+      <c r="AJ10">
+        <v>67.180000000000007</v>
+      </c>
+      <c r="AK10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL10">
+        <v>80.017974835230675</v>
+      </c>
+      <c r="AM10">
+        <v>77.980826842420612</v>
+      </c>
+      <c r="AN10">
+        <v>62.402636309167171</v>
+      </c>
+      <c r="AO10">
+        <v>77.980826842420612</v>
+      </c>
+      <c r="AP10">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>9</v>
       </c>
       <c r="B11">
-        <v>14</v>
+        <v>70</v>
       </c>
       <c r="C11" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="D11">
-        <v>1431</v>
+        <v>-3452</v>
       </c>
       <c r="E11">
-        <v>70.099999999999994</v>
+        <v>76.98</v>
       </c>
       <c r="F11" t="b">
         <v>1</v>
       </c>
       <c r="G11">
-        <v>1347.4841916191081</v>
+        <v>-3541.0518878509738</v>
       </c>
       <c r="H11">
-        <v>383.82581561085141</v>
+        <v>417.98388959163412</v>
       </c>
       <c r="I11">
         <v>100</v>
       </c>
       <c r="J11" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="K11" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="L11">
-        <v>1694</v>
+        <v>-1146</v>
       </c>
       <c r="M11">
-        <v>71.600000000000009</v>
+        <v>70.27000000000001</v>
       </c>
       <c r="N11" t="b">
         <v>1</v>
       </c>
       <c r="O11" t="s">
-        <v>65</v>
-      </c>
-      <c r="P11">
-        <v>-1701</v>
+        <v>71</v>
+      </c>
+      <c r="P11" t="s">
+        <v>72</v>
       </c>
       <c r="Q11">
-        <v>69.300000000000011</v>
+        <v>0</v>
       </c>
       <c r="R11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S11" t="s">
-        <v>65</v>
-      </c>
-      <c r="T11">
-        <v>-1701</v>
+        <v>71</v>
+      </c>
+      <c r="T11" t="s">
+        <v>72</v>
       </c>
       <c r="U11">
-        <v>69.300000000000011</v>
+        <v>0</v>
       </c>
       <c r="V11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W11" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="X11" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="Y11">
-        <v>1372</v>
+        <v>-1146</v>
       </c>
       <c r="Z11">
-        <v>75.3</v>
+        <v>70.27000000000001</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
       </c>
-      <c r="AB11">
-        <v>15.52538370720189</v>
-      </c>
-      <c r="AC11">
-        <v>200.41322314049589</v>
-      </c>
-      <c r="AD11">
-        <v>200.41322314049589</v>
-      </c>
-      <c r="AE11">
-        <v>19.008264462809919</v>
-      </c>
-    </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.3">
-      <c r="AB13">
-        <f>AVERAGE(AB2:AB11)</f>
-        <v>18.404815167539788</v>
-      </c>
-      <c r="AC13">
-        <f t="shared" ref="AC13:AE13" si="0">AVERAGE(AC2:AC11)</f>
-        <v>72.78505781225283</v>
-      </c>
-      <c r="AD13">
-        <f t="shared" si="0"/>
-        <v>69.53421529049497</v>
-      </c>
-      <c r="AE13">
-        <f t="shared" si="0"/>
-        <v>5.9363425558543295</v>
+      <c r="AB11" t="s">
+        <v>73</v>
+      </c>
+      <c r="AD11" t="s">
+        <v>72</v>
+      </c>
+      <c r="AE11" t="s">
+        <v>74</v>
+      </c>
+      <c r="AF11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AG11" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH11" t="s">
+        <v>75</v>
+      </c>
+      <c r="AI11">
+        <v>-1953</v>
+      </c>
+      <c r="AJ11">
+        <v>76.2</v>
+      </c>
+      <c r="AK11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL11">
+        <v>201.22164048865619</v>
       </c>
     </row>
   </sheetData>
@@ -1727,65 +2083,77 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>75</v>
+        <v>84</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>86</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="B2">
         <v>10</v>
       </c>
       <c r="C2">
-        <v>4412.1000000000004</v>
+        <v>3016.4</v>
       </c>
       <c r="D2">
-        <v>3563</v>
+        <v>1239.9000000000001</v>
       </c>
       <c r="E2">
-        <v>1722.2</v>
+        <v>2897.7777777777778</v>
       </c>
       <c r="F2">
-        <v>1854.6</v>
+        <v>2962.4444444444439</v>
       </c>
       <c r="G2">
-        <v>4188.3</v>
+        <v>2891.7</v>
       </c>
       <c r="H2">
-        <v>4685.402284860611</v>
+        <v>2897.7777777777778</v>
       </c>
       <c r="I2">
-        <v>18.404815167539791</v>
+        <v>2935.7</v>
+      </c>
+      <c r="J2">
+        <v>2275.3471717834468</v>
+      </c>
+      <c r="K2">
+        <v>63.327122592051587</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Eliminacion de max steps per episode, version mas estable AM-PPO  y avg GAP de 21%.
</commit_message>
<xml_diff>
--- a/DRL_Routing_Summary_stochastic_sigma10%_AM.xlsx
+++ b/DRL_Routing_Summary_stochastic_sigma10%_AM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a9faf7a5fe1343c6/Desktop/Maestria/Tesis MSc/RoutingModel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_8B418FE7927CD14D70B4967629358AD3C21C49B1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4DB17FA8-C42A-43BA-A53B-3BBAA1D189FA}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="11_8B418FE71B54906DBDD3C5B532358AD3C21C4A92" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{41281C83-72D8-42E5-9F56-9A25540FB4C2}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="88">
   <si>
     <t>Start Node</t>
   </si>
@@ -158,7 +158,7 @@
     <t>Optimal</t>
   </si>
   <si>
-    <t>[0, 1, 2, 6, 0]</t>
+    <t>[0, 1, 2, 0]</t>
   </si>
   <si>
     <t>[0, 2, 1, 0]</t>
@@ -167,106 +167,88 @@
     <t>[1, 0, 6, 7, 1]</t>
   </si>
   <si>
-    <t>[1, 6, 0, 2, 1]</t>
-  </si>
-  <si>
-    <t>[1, 2, 8, 0, 6, 1]</t>
-  </si>
-  <si>
-    <t>[1, 6, 2, 8, 0, 1]</t>
+    <t>[1, 0, 2, 8, 1]</t>
+  </si>
+  <si>
+    <t>[1, 2, 8, 6, 1]</t>
+  </si>
+  <si>
+    <t>[1, 6, 7, 8, 1]</t>
+  </si>
+  <si>
+    <t>[2, 6, 7, 8, 2]</t>
+  </si>
+  <si>
+    <t>[2, 8, 7, 6, 2]</t>
+  </si>
+  <si>
+    <t>[2, 4, 2]</t>
+  </si>
+  <si>
+    <t>[3, 4, 5, 3]</t>
+  </si>
+  <si>
+    <t>[3, 5, 4, 3]</t>
+  </si>
+  <si>
+    <t>[4, 2, 4]</t>
+  </si>
+  <si>
+    <t>[4, 8, 2, 4]</t>
+  </si>
+  <si>
+    <t>[5, 3, 5]</t>
+  </si>
+  <si>
+    <t>[5, 4, 3, 5]</t>
+  </si>
+  <si>
+    <t>[6, 0, 1, 7, 6]</t>
+  </si>
+  <si>
+    <t>[6, 2, 8, 1, 6]</t>
+  </si>
+  <si>
+    <t>[6, 2, 1, 6]</t>
+  </si>
+  <si>
+    <t>[7, 6, 2, 7]</t>
+  </si>
+  <si>
+    <t>[7, 2, 6, 7]</t>
+  </si>
+  <si>
+    <t>[8, 0, 6, 8]</t>
+  </si>
+  <si>
+    <t>[8, 2, 1, 0, 8]</t>
+  </si>
+  <si>
+    <t>[8, 1, 2, 8]</t>
+  </si>
+  <si>
+    <t>[8, 1, 0, 2, 8]</t>
+  </si>
+  <si>
+    <t>[9, 6, 1, 9]</t>
+  </si>
+  <si>
+    <t>[9, 1, 6, 9]</t>
+  </si>
+  <si>
+    <t>[9]</t>
+  </si>
+  <si>
+    <t>-inf</t>
+  </si>
+  <si>
+    <t>[9, 2, 8, 1, 9]</t>
   </si>
   <si>
     <t>Infeasible</t>
   </si>
   <si>
-    <t>-inf</t>
-  </si>
-  <si>
     <t>inf</t>
-  </si>
-  <si>
-    <t>[2, 1, 0, 6, 2]</t>
-  </si>
-  <si>
-    <t>[2, 7, 6, 0, 2]</t>
-  </si>
-  <si>
-    <t>[2, 5, 2]</t>
-  </si>
-  <si>
-    <t>[3, 5, 3]</t>
-  </si>
-  <si>
-    <t>[3, 5, 4, 3]</t>
-  </si>
-  <si>
-    <t>[3, 2, 4, 3]</t>
-  </si>
-  <si>
-    <t>[4, 2, 4]</t>
-  </si>
-  <si>
-    <t>[4, 3, 2, 4]</t>
-  </si>
-  <si>
-    <t>[4, 5, 3, 4]</t>
-  </si>
-  <si>
-    <t>[4, 1, 2, 4]</t>
-  </si>
-  <si>
-    <t>[5, 4, 3, 5]</t>
-  </si>
-  <si>
-    <t>[5, 3, 4, 5]</t>
-  </si>
-  <si>
-    <t>[6, 2, 8, 0, 6]</t>
-  </si>
-  <si>
-    <t>[6, 0, 2, 7, 6]</t>
-  </si>
-  <si>
-    <t>[6, 2, 7, 6]</t>
-  </si>
-  <si>
-    <t>[7, 0, 6, 1, 7]</t>
-  </si>
-  <si>
-    <t>[7, 6, 1, 2, 7]</t>
-  </si>
-  <si>
-    <t>[7, 1, 2, 8, 7]</t>
-  </si>
-  <si>
-    <t>[8, 7, 0, 6, 8]</t>
-  </si>
-  <si>
-    <t>[8, 2, 6, 0, 8]</t>
-  </si>
-  <si>
-    <t>[8, 1, 2, 6, 8]</t>
-  </si>
-  <si>
-    <t>[8, 6, 2, 1, 8]</t>
-  </si>
-  <si>
-    <t>[8, 1, 6, 0, 8]</t>
-  </si>
-  <si>
-    <t>[8, 2, 1, 0, 8]</t>
-  </si>
-  <si>
-    <t>[9, 2, 8, 9]</t>
-  </si>
-  <si>
-    <t>[9, 1, 6, 2, 9]</t>
-  </si>
-  <si>
-    <t>[9]</t>
-  </si>
-  <si>
-    <t>[9, 8, 1, 2, 9]</t>
   </si>
   <si>
     <t>Model</t>
@@ -668,8 +650,19 @@
   <dimension ref="A1:AQ11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="14.6640625" customWidth="1"/>
-    <col min="4" max="4" width="18.33203125" customWidth="1"/>
+    <col min="3" max="3" width="15.44140625" customWidth="1"/>
+    <col min="11" max="11" width="14.44140625" customWidth="1"/>
+    <col min="15" max="15" width="15.44140625" customWidth="1"/>
+    <col min="19" max="19" width="15.5546875" customWidth="1"/>
+    <col min="24" max="24" width="15.6640625" customWidth="1"/>
+    <col min="29" max="29" width="15.33203125" customWidth="1"/>
+    <col min="34" max="34" width="14" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="17.5546875" customWidth="1"/>
+    <col min="39" max="39" width="18.44140625" customWidth="1"/>
+    <col min="40" max="40" width="15.109375" customWidth="1"/>
+    <col min="41" max="41" width="15" customWidth="1"/>
+    <col min="42" max="42" width="16.33203125" customWidth="1"/>
+    <col min="43" max="43" width="19" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:43" x14ac:dyDescent="0.3">
@@ -817,7 +810,7 @@
         <v>2403</v>
       </c>
       <c r="E2">
-        <v>58.09</v>
+        <v>74.09</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
@@ -838,10 +831,10 @@
         <v>45</v>
       </c>
       <c r="L2">
-        <v>4273</v>
+        <v>3424</v>
       </c>
       <c r="M2">
-        <v>63.05</v>
+        <v>68.25</v>
       </c>
       <c r="N2" t="b">
         <v>1</v>
@@ -853,7 +846,7 @@
         <v>3275</v>
       </c>
       <c r="Q2">
-        <v>56.179999999999993</v>
+        <v>68.179999999999993</v>
       </c>
       <c r="R2" t="b">
         <v>1</v>
@@ -862,10 +855,10 @@
         <v>45</v>
       </c>
       <c r="T2">
-        <v>4273</v>
+        <v>3424</v>
       </c>
       <c r="U2">
-        <v>63.05</v>
+        <v>68.25</v>
       </c>
       <c r="V2" t="b">
         <v>1</v>
@@ -877,10 +870,10 @@
         <v>45</v>
       </c>
       <c r="Y2">
-        <v>4273</v>
+        <v>3424</v>
       </c>
       <c r="Z2">
-        <v>63.05</v>
+        <v>68.25</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -895,7 +888,7 @@
         <v>3275</v>
       </c>
       <c r="AE2">
-        <v>56.179999999999993</v>
+        <v>68.179999999999993</v>
       </c>
       <c r="AF2" t="b">
         <v>1</v>
@@ -907,19 +900,19 @@
         <v>45</v>
       </c>
       <c r="AI2">
-        <v>4273</v>
+        <v>3424</v>
       </c>
       <c r="AJ2">
-        <v>63.05</v>
+        <v>68.25</v>
       </c>
       <c r="AK2" t="b">
         <v>1</v>
       </c>
       <c r="AL2">
-        <v>43.763164053358302</v>
+        <v>29.818925233644858</v>
       </c>
       <c r="AM2">
-        <v>23.35595600280833</v>
+        <v>4.3516355140186924</v>
       </c>
       <c r="AN2">
         <v>0</v>
@@ -928,7 +921,7 @@
         <v>0</v>
       </c>
       <c r="AP2">
-        <v>23.35595600280833</v>
+        <v>4.3516355140186924</v>
       </c>
       <c r="AQ2">
         <v>0</v>
@@ -939,25 +932,25 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>40</v>
+        <v>61</v>
       </c>
       <c r="C3" t="s">
         <v>47</v>
       </c>
       <c r="D3">
-        <v>3653</v>
+        <v>3284</v>
       </c>
       <c r="E3">
-        <v>58.09</v>
+        <v>74.09</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
       </c>
       <c r="G3">
-        <v>3668.2358799880622</v>
+        <v>3416.1097767738888</v>
       </c>
       <c r="H3">
-        <v>500.73301317621241</v>
+        <v>430.07934961368261</v>
       </c>
       <c r="I3">
         <v>100</v>
@@ -969,10 +962,10 @@
         <v>48</v>
       </c>
       <c r="L3">
-        <v>4352</v>
+        <v>4600</v>
       </c>
       <c r="M3">
-        <v>72.849999999999994</v>
+        <v>76.949999999999989</v>
       </c>
       <c r="N3" t="b">
         <v>1</v>
@@ -981,22 +974,22 @@
         <v>49</v>
       </c>
       <c r="P3">
-        <v>2026</v>
+        <v>1661</v>
       </c>
       <c r="Q3">
-        <v>76.349999999999994</v>
+        <v>66.38</v>
       </c>
       <c r="R3" t="b">
         <v>1</v>
       </c>
       <c r="S3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="T3">
-        <v>4381</v>
+        <v>1661</v>
       </c>
       <c r="U3">
-        <v>76.48</v>
+        <v>66.38</v>
       </c>
       <c r="V3" t="b">
         <v>1</v>
@@ -1008,58 +1001,61 @@
         <v>48</v>
       </c>
       <c r="Y3">
-        <v>4352</v>
+        <v>4600</v>
       </c>
       <c r="Z3">
-        <v>72.849999999999994</v>
+        <v>76.949999999999989</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
       </c>
       <c r="AB3" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="AC3" t="s">
         <v>49</v>
       </c>
-      <c r="AD3" t="s">
-        <v>52</v>
-      </c>
-      <c r="AE3" t="s">
-        <v>53</v>
+      <c r="AD3">
+        <v>1661</v>
+      </c>
+      <c r="AE3">
+        <v>66.38</v>
       </c>
       <c r="AF3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG3" t="s">
         <v>44</v>
       </c>
       <c r="AH3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="AI3">
-        <v>4352</v>
+        <v>3987</v>
       </c>
       <c r="AJ3">
-        <v>72.849999999999994</v>
+        <v>73.150000000000006</v>
       </c>
       <c r="AK3" t="b">
         <v>1</v>
       </c>
       <c r="AL3">
-        <v>16.061580882352938</v>
+        <v>28.60869565217391</v>
       </c>
       <c r="AM3">
-        <v>53.446691176470587</v>
+        <v>63.891304347826093</v>
       </c>
       <c r="AN3">
-        <v>-0.66636029411764708</v>
+        <v>63.891304347826093</v>
       </c>
       <c r="AO3">
         <v>0</v>
       </c>
+      <c r="AP3">
+        <v>63.891304347826093</v>
+      </c>
       <c r="AQ3">
-        <v>0</v>
+        <v>13.32608695652174</v>
       </c>
     </row>
     <row r="4" spans="1:43" x14ac:dyDescent="0.3">
@@ -1067,25 +1063,25 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>10</v>
+        <v>82</v>
       </c>
       <c r="C4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D4">
-        <v>691</v>
+        <v>3942</v>
       </c>
       <c r="E4">
-        <v>63.05</v>
+        <v>70.449999999999989</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
       </c>
       <c r="G4">
-        <v>705.99961675565544</v>
+        <v>3983.0152287408432</v>
       </c>
       <c r="H4">
-        <v>387.97063498656439</v>
+        <v>419.55948863432269</v>
       </c>
       <c r="I4">
         <v>100</v>
@@ -1094,37 +1090,37 @@
         <v>44</v>
       </c>
       <c r="K4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="L4">
-        <v>2814</v>
+        <v>3942</v>
       </c>
       <c r="M4">
-        <v>76.94</v>
+        <v>70.45</v>
       </c>
       <c r="N4" t="b">
         <v>1</v>
       </c>
       <c r="O4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="P4">
-        <v>-1212</v>
+        <v>1834</v>
       </c>
       <c r="Q4">
-        <v>73.8</v>
+        <v>55.8</v>
       </c>
       <c r="R4" t="b">
         <v>1</v>
       </c>
       <c r="S4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="T4">
-        <v>-1212</v>
+        <v>1834</v>
       </c>
       <c r="U4">
-        <v>73.8</v>
+        <v>55.8</v>
       </c>
       <c r="V4" t="b">
         <v>1</v>
@@ -1133,13 +1129,13 @@
         <v>44</v>
       </c>
       <c r="X4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="Y4">
-        <v>2814</v>
+        <v>3942</v>
       </c>
       <c r="Z4">
-        <v>76.94</v>
+        <v>70.449999999999989</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -1148,13 +1144,13 @@
         <v>44</v>
       </c>
       <c r="AC4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="AD4">
-        <v>-1212</v>
+        <v>1834</v>
       </c>
       <c r="AE4">
-        <v>73.8</v>
+        <v>55.8</v>
       </c>
       <c r="AF4" t="b">
         <v>1</v>
@@ -1163,31 +1159,31 @@
         <v>44</v>
       </c>
       <c r="AH4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="AI4">
-        <v>2814</v>
+        <v>3942</v>
       </c>
       <c r="AJ4">
-        <v>76.94</v>
+        <v>70.449999999999989</v>
       </c>
       <c r="AK4" t="b">
         <v>1</v>
       </c>
       <c r="AL4">
-        <v>75.44420753375978</v>
+        <v>0</v>
       </c>
       <c r="AM4">
-        <v>143.07036247334759</v>
+        <v>53.475393201420587</v>
       </c>
       <c r="AN4">
-        <v>143.07036247334759</v>
+        <v>53.475393201420587</v>
       </c>
       <c r="AO4">
         <v>0</v>
       </c>
       <c r="AP4">
-        <v>143.07036247334759</v>
+        <v>53.475393201420587</v>
       </c>
       <c r="AQ4">
         <v>0</v>
@@ -1198,25 +1194,25 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>65</v>
+        <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D5">
-        <v>862</v>
+        <v>1886</v>
       </c>
       <c r="E5">
-        <v>26.24</v>
+        <v>54.16</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>839.548651744719</v>
+        <v>1946.1447474123879</v>
       </c>
       <c r="H5">
-        <v>289.357081943732</v>
+        <v>373.16155105572739</v>
       </c>
       <c r="I5">
         <v>100</v>
@@ -1225,37 +1221,37 @@
         <v>44</v>
       </c>
       <c r="K5" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="L5">
-        <v>2423</v>
+        <v>1886</v>
       </c>
       <c r="M5">
-        <v>42.16</v>
+        <v>54.16</v>
       </c>
       <c r="N5" t="b">
         <v>1</v>
       </c>
       <c r="O5" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="P5">
-        <v>2209</v>
+        <v>1886</v>
       </c>
       <c r="Q5">
-        <v>68.070000000000007</v>
+        <v>54.16</v>
       </c>
       <c r="R5" t="b">
         <v>1</v>
       </c>
       <c r="S5" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="T5">
-        <v>2209</v>
+        <v>1886</v>
       </c>
       <c r="U5">
-        <v>68.070000000000007</v>
+        <v>54.16</v>
       </c>
       <c r="V5" t="b">
         <v>1</v>
@@ -1264,13 +1260,13 @@
         <v>44</v>
       </c>
       <c r="X5" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="Y5">
-        <v>2423</v>
+        <v>1886</v>
       </c>
       <c r="Z5">
-        <v>42.16</v>
+        <v>54.16</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1279,13 +1275,13 @@
         <v>44</v>
       </c>
       <c r="AC5" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="AD5">
-        <v>2209</v>
+        <v>1886</v>
       </c>
       <c r="AE5">
-        <v>68.070000000000007</v>
+        <v>54.16</v>
       </c>
       <c r="AF5" t="b">
         <v>1</v>
@@ -1294,31 +1290,31 @@
         <v>44</v>
       </c>
       <c r="AH5" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="AI5">
-        <v>2423</v>
+        <v>1886</v>
       </c>
       <c r="AJ5">
-        <v>42.16</v>
+        <v>54.16</v>
       </c>
       <c r="AK5" t="b">
         <v>1</v>
       </c>
       <c r="AL5">
-        <v>64.424267437061488</v>
+        <v>0</v>
       </c>
       <c r="AM5">
-        <v>8.8320264135369371</v>
+        <v>0</v>
       </c>
       <c r="AN5">
-        <v>8.8320264135369371</v>
+        <v>0</v>
       </c>
       <c r="AO5">
         <v>0</v>
       </c>
       <c r="AP5">
-        <v>8.8320264135369371</v>
+        <v>0</v>
       </c>
       <c r="AQ5">
         <v>0</v>
@@ -1329,25 +1325,25 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="C6" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D6">
-        <v>3491</v>
+        <v>2006</v>
       </c>
       <c r="E6">
-        <v>47.8</v>
+        <v>55.8</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
       </c>
       <c r="G6">
-        <v>3453.126181562021</v>
+        <v>1988.8867739611539</v>
       </c>
       <c r="H6">
-        <v>270.34065861475818</v>
+        <v>248.96790977144721</v>
       </c>
       <c r="I6">
         <v>100</v>
@@ -1356,37 +1352,37 @@
         <v>44</v>
       </c>
       <c r="K6" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="L6">
-        <v>3832</v>
+        <v>2487</v>
       </c>
       <c r="M6">
-        <v>68.070000000000007</v>
+        <v>72.3</v>
       </c>
       <c r="N6" t="b">
         <v>1</v>
       </c>
       <c r="O6" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="P6">
-        <v>2004</v>
+        <v>2487</v>
       </c>
       <c r="Q6">
-        <v>42.15</v>
+        <v>72.3</v>
       </c>
       <c r="R6" t="b">
         <v>1</v>
       </c>
       <c r="S6" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="T6">
-        <v>2004</v>
+        <v>2487</v>
       </c>
       <c r="U6">
-        <v>42.15</v>
+        <v>72.3</v>
       </c>
       <c r="V6" t="b">
         <v>1</v>
@@ -1395,13 +1391,13 @@
         <v>44</v>
       </c>
       <c r="X6" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="Y6">
-        <v>3832</v>
+        <v>2487</v>
       </c>
       <c r="Z6">
-        <v>68.070000000000007</v>
+        <v>72.3</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1410,13 +1406,13 @@
         <v>44</v>
       </c>
       <c r="AC6" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="AD6">
-        <v>2004</v>
+        <v>2487</v>
       </c>
       <c r="AE6">
-        <v>42.15</v>
+        <v>72.3</v>
       </c>
       <c r="AF6" t="b">
         <v>1</v>
@@ -1425,34 +1421,34 @@
         <v>44</v>
       </c>
       <c r="AH6" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="AI6">
-        <v>3683</v>
+        <v>2487</v>
       </c>
       <c r="AJ6">
-        <v>76.709999999999994</v>
+        <v>72.3</v>
       </c>
       <c r="AK6" t="b">
         <v>1</v>
       </c>
       <c r="AL6">
-        <v>8.8987473903966592</v>
+        <v>19.340570969039</v>
       </c>
       <c r="AM6">
-        <v>47.703549060542798</v>
+        <v>0</v>
       </c>
       <c r="AN6">
-        <v>47.703549060542798</v>
+        <v>0</v>
       </c>
       <c r="AO6">
         <v>0</v>
       </c>
       <c r="AP6">
-        <v>47.703549060542798</v>
+        <v>0</v>
       </c>
       <c r="AQ6">
-        <v>3.8883089770354911</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:43" x14ac:dyDescent="0.3">
@@ -1460,25 +1456,25 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="C7" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="D7">
-        <v>2004</v>
+        <v>1008</v>
       </c>
       <c r="E7">
-        <v>42.15</v>
+        <v>34.239999999999988</v>
       </c>
       <c r="F7" t="b">
         <v>1</v>
       </c>
       <c r="G7">
-        <v>2076.0753950047092</v>
+        <v>1026.6930563382371</v>
       </c>
       <c r="H7">
-        <v>418.72686703177021</v>
+        <v>292.34118593450211</v>
       </c>
       <c r="I7">
         <v>100</v>
@@ -1487,37 +1483,37 @@
         <v>44</v>
       </c>
       <c r="K7" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="L7">
-        <v>2004</v>
+        <v>2183</v>
       </c>
       <c r="M7">
-        <v>42.15</v>
+        <v>54.16</v>
       </c>
       <c r="N7" t="b">
         <v>1</v>
       </c>
       <c r="O7" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="P7">
-        <v>2004</v>
+        <v>2183</v>
       </c>
       <c r="Q7">
-        <v>42.15</v>
+        <v>54.16</v>
       </c>
       <c r="R7" t="b">
         <v>1</v>
       </c>
       <c r="S7" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="T7">
-        <v>2004</v>
+        <v>2183</v>
       </c>
       <c r="U7">
-        <v>42.15</v>
+        <v>54.16</v>
       </c>
       <c r="V7" t="b">
         <v>1</v>
@@ -1526,13 +1522,13 @@
         <v>44</v>
       </c>
       <c r="X7" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="Y7">
-        <v>2004</v>
+        <v>2183</v>
       </c>
       <c r="Z7">
-        <v>42.15</v>
+        <v>54.16</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1541,13 +1537,13 @@
         <v>44</v>
       </c>
       <c r="AC7" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="AD7">
-        <v>2004</v>
+        <v>2183</v>
       </c>
       <c r="AE7">
-        <v>42.15</v>
+        <v>54.16</v>
       </c>
       <c r="AF7" t="b">
         <v>1</v>
@@ -1556,19 +1552,19 @@
         <v>44</v>
       </c>
       <c r="AH7" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="AI7">
-        <v>2004</v>
+        <v>2183</v>
       </c>
       <c r="AJ7">
-        <v>42.15</v>
+        <v>54.16</v>
       </c>
       <c r="AK7" t="b">
         <v>1</v>
       </c>
       <c r="AL7">
-        <v>0</v>
+        <v>53.825011452130099</v>
       </c>
       <c r="AM7">
         <v>0</v>
@@ -1591,25 +1587,25 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>65</v>
+        <v>34</v>
       </c>
       <c r="C8" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D8">
-        <v>4252</v>
+        <v>3449</v>
       </c>
       <c r="E8">
-        <v>64.510000000000005</v>
+        <v>74.59</v>
       </c>
       <c r="F8" t="b">
         <v>1</v>
       </c>
       <c r="G8">
-        <v>4381.1768970787016</v>
+        <v>3443.7589494943331</v>
       </c>
       <c r="H8">
-        <v>385.04831990271379</v>
+        <v>391.10814814573399</v>
       </c>
       <c r="I8">
         <v>100</v>
@@ -1618,37 +1614,37 @@
         <v>44</v>
       </c>
       <c r="K8" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="L8">
-        <v>4788</v>
+        <v>4842</v>
       </c>
       <c r="M8">
-        <v>76.94</v>
+        <v>71.099999999999994</v>
       </c>
       <c r="N8" t="b">
         <v>1</v>
       </c>
       <c r="O8" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="P8">
-        <v>3610</v>
+        <v>4691</v>
       </c>
       <c r="Q8">
-        <v>54.419999999999987</v>
+        <v>62.33</v>
       </c>
       <c r="R8" t="b">
         <v>1</v>
       </c>
       <c r="S8" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="T8">
-        <v>4788</v>
+        <v>4842</v>
       </c>
       <c r="U8">
-        <v>76.94</v>
+        <v>71.099999999999994</v>
       </c>
       <c r="V8" t="b">
         <v>1</v>
@@ -1657,13 +1653,13 @@
         <v>44</v>
       </c>
       <c r="X8" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="Y8">
-        <v>4788</v>
+        <v>4691</v>
       </c>
       <c r="Z8">
-        <v>76.94</v>
+        <v>62.33</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1672,13 +1668,13 @@
         <v>44</v>
       </c>
       <c r="AC8" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="AD8">
-        <v>3610</v>
+        <v>4691</v>
       </c>
       <c r="AE8">
-        <v>54.419999999999987</v>
+        <v>62.33</v>
       </c>
       <c r="AF8" t="b">
         <v>1</v>
@@ -1687,34 +1683,34 @@
         <v>44</v>
       </c>
       <c r="AH8" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="AI8">
-        <v>4788</v>
+        <v>4691</v>
       </c>
       <c r="AJ8">
-        <v>76.94</v>
+        <v>62.33</v>
       </c>
       <c r="AK8" t="b">
         <v>1</v>
       </c>
       <c r="AL8">
-        <v>11.19465329991646</v>
+        <v>28.769103676166871</v>
       </c>
       <c r="AM8">
-        <v>24.603174603174601</v>
+        <v>3.1185460553490292</v>
       </c>
       <c r="AN8">
         <v>0</v>
       </c>
       <c r="AO8">
-        <v>0</v>
+        <v>3.1185460553490292</v>
       </c>
       <c r="AP8">
-        <v>24.603174603174601</v>
+        <v>3.1185460553490292</v>
       </c>
       <c r="AQ8">
-        <v>0</v>
+        <v>3.1185460553490292</v>
       </c>
     </row>
     <row r="9" spans="1:43" x14ac:dyDescent="0.3">
@@ -1722,25 +1718,25 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="C9" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="D9">
-        <v>3848</v>
+        <v>3681</v>
       </c>
       <c r="E9">
-        <v>74.17</v>
+        <v>66.430000000000007</v>
       </c>
       <c r="F9" t="b">
         <v>1</v>
       </c>
       <c r="G9">
-        <v>4008.006328774984</v>
+        <v>3676.3394265887018</v>
       </c>
       <c r="H9">
-        <v>408.8562102122832</v>
+        <v>367.94400640819322</v>
       </c>
       <c r="I9">
         <v>100</v>
@@ -1749,37 +1745,37 @@
         <v>44</v>
       </c>
       <c r="K9" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="L9">
-        <v>4235</v>
+        <v>3681</v>
       </c>
       <c r="M9">
-        <v>65.75</v>
+        <v>66.430000000000007</v>
       </c>
       <c r="N9" t="b">
         <v>1</v>
       </c>
       <c r="O9" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="P9">
-        <v>3224</v>
+        <v>3681</v>
       </c>
       <c r="Q9">
-        <v>65.28</v>
+        <v>66.430000000000007</v>
       </c>
       <c r="R9" t="b">
         <v>1</v>
       </c>
       <c r="S9" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="T9">
-        <v>3224</v>
+        <v>3681</v>
       </c>
       <c r="U9">
-        <v>65.28</v>
+        <v>66.430000000000007</v>
       </c>
       <c r="V9" t="b">
         <v>1</v>
@@ -1788,13 +1784,13 @@
         <v>44</v>
       </c>
       <c r="X9" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="Y9">
-        <v>4235</v>
+        <v>3681</v>
       </c>
       <c r="Z9">
-        <v>65.75</v>
+        <v>66.430000000000007</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1803,13 +1799,13 @@
         <v>44</v>
       </c>
       <c r="AC9" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="AD9">
-        <v>3224</v>
+        <v>3681</v>
       </c>
       <c r="AE9">
-        <v>65.28</v>
+        <v>66.430000000000007</v>
       </c>
       <c r="AF9" t="b">
         <v>1</v>
@@ -1818,31 +1814,31 @@
         <v>44</v>
       </c>
       <c r="AH9" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="AI9">
-        <v>4235</v>
+        <v>3681</v>
       </c>
       <c r="AJ9">
-        <v>65.75</v>
+        <v>66.430000000000007</v>
       </c>
       <c r="AK9" t="b">
         <v>1</v>
       </c>
       <c r="AL9">
-        <v>9.1381345926800464</v>
+        <v>0</v>
       </c>
       <c r="AM9">
-        <v>23.872491145218419</v>
+        <v>0</v>
       </c>
       <c r="AN9">
-        <v>23.872491145218419</v>
+        <v>0</v>
       </c>
       <c r="AO9">
         <v>0</v>
       </c>
       <c r="AP9">
-        <v>23.872491145218419</v>
+        <v>0</v>
       </c>
       <c r="AQ9">
         <v>0</v>
@@ -1853,25 +1849,25 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>79</v>
+        <v>0</v>
       </c>
       <c r="C10" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="D10">
-        <v>3656</v>
+        <v>1742</v>
       </c>
       <c r="E10">
-        <v>69.89</v>
+        <v>63.13000000000001</v>
       </c>
       <c r="F10" t="b">
         <v>1</v>
       </c>
       <c r="G10">
-        <v>3706.2492956588562</v>
+        <v>1770.757128269227</v>
       </c>
       <c r="H10">
-        <v>402.18560383717909</v>
+        <v>363.11846402797357</v>
       </c>
       <c r="I10">
         <v>100</v>
@@ -1880,37 +1876,37 @@
         <v>44</v>
       </c>
       <c r="K10" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="L10">
-        <v>4148</v>
+        <v>3415</v>
       </c>
       <c r="M10">
-        <v>64.510000000000005</v>
+        <v>75.17</v>
       </c>
       <c r="N10" t="b">
         <v>1</v>
       </c>
       <c r="O10" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="P10">
-        <v>1648</v>
+        <v>2383</v>
       </c>
       <c r="Q10">
-        <v>63.43</v>
+        <v>49.81</v>
       </c>
       <c r="R10" t="b">
         <v>1</v>
       </c>
       <c r="S10" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="T10">
-        <v>1750</v>
+        <v>3257</v>
       </c>
       <c r="U10">
-        <v>63.03</v>
+        <v>76.949999999999989</v>
       </c>
       <c r="V10" t="b">
         <v>1</v>
@@ -1919,13 +1915,13 @@
         <v>44</v>
       </c>
       <c r="X10" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="Y10">
-        <v>3756</v>
+        <v>3415</v>
       </c>
       <c r="Z10">
-        <v>67.180000000000007</v>
+        <v>75.17</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1934,13 +1930,13 @@
         <v>44</v>
       </c>
       <c r="AC10" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="AD10">
-        <v>1648</v>
+        <v>2383</v>
       </c>
       <c r="AE10">
-        <v>63.43</v>
+        <v>49.81</v>
       </c>
       <c r="AF10" t="b">
         <v>1</v>
@@ -1949,34 +1945,34 @@
         <v>44</v>
       </c>
       <c r="AH10" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="AI10">
-        <v>3285</v>
+        <v>3415</v>
       </c>
       <c r="AJ10">
-        <v>59.17</v>
+        <v>75.17</v>
       </c>
       <c r="AK10" t="b">
         <v>1</v>
       </c>
       <c r="AL10">
-        <v>11.86113789778206</v>
+        <v>48.989751098096633</v>
       </c>
       <c r="AM10">
-        <v>60.27000964320154</v>
+        <v>30.21961932650073</v>
       </c>
       <c r="AN10">
-        <v>57.810993249758923</v>
+        <v>4.6266471449487554</v>
       </c>
       <c r="AO10">
-        <v>9.4503375120540021</v>
+        <v>0</v>
       </c>
       <c r="AP10">
-        <v>60.27000964320154</v>
+        <v>30.21961932650073</v>
       </c>
       <c r="AQ10">
-        <v>20.80520732883317</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:43" x14ac:dyDescent="0.3">
@@ -1984,25 +1980,25 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C11" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="D11">
-        <v>-352</v>
+        <v>788</v>
       </c>
       <c r="E11">
-        <v>47.53</v>
+        <v>76.650000000000006</v>
       </c>
       <c r="F11" t="b">
         <v>1</v>
       </c>
       <c r="G11">
-        <v>-468.38734132249971</v>
+        <v>720.80446795516764</v>
       </c>
       <c r="H11">
-        <v>343.61833480578429</v>
+        <v>354.89192131506701</v>
       </c>
       <c r="I11">
         <v>100</v>
@@ -2011,22 +2007,22 @@
         <v>44</v>
       </c>
       <c r="K11" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="L11">
-        <v>1170</v>
+        <v>788</v>
       </c>
       <c r="M11">
-        <v>70.349999999999994</v>
+        <v>76.650000000000006</v>
       </c>
       <c r="N11" t="b">
         <v>1</v>
       </c>
       <c r="O11" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="P11" t="s">
-        <v>52</v>
+        <v>72</v>
       </c>
       <c r="Q11">
         <v>0</v>
@@ -2035,10 +2031,10 @@
         <v>0</v>
       </c>
       <c r="S11" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="T11" t="s">
-        <v>52</v>
+        <v>72</v>
       </c>
       <c r="U11">
         <v>0</v>
@@ -2050,25 +2046,25 @@
         <v>44</v>
       </c>
       <c r="X11" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="Y11">
-        <v>1080</v>
+        <v>-1836</v>
       </c>
       <c r="Z11">
-        <v>71.91</v>
+        <v>73.75</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
       </c>
       <c r="AB11" t="s">
-        <v>51</v>
+        <v>74</v>
       </c>
       <c r="AD11" t="s">
-        <v>52</v>
+        <v>72</v>
       </c>
       <c r="AE11" t="s">
-        <v>53</v>
+        <v>75</v>
       </c>
       <c r="AF11" t="b">
         <v>0</v>
@@ -2077,25 +2073,25 @@
         <v>44</v>
       </c>
       <c r="AH11" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="AI11">
-        <v>1080</v>
+        <v>-1836</v>
       </c>
       <c r="AJ11">
-        <v>71.91</v>
+        <v>73.75</v>
       </c>
       <c r="AK11" t="b">
         <v>1</v>
       </c>
       <c r="AL11">
-        <v>130.08547008547009</v>
+        <v>0</v>
       </c>
       <c r="AO11">
-        <v>7.6923076923076934</v>
+        <v>332.99492385786812</v>
       </c>
       <c r="AQ11">
-        <v>7.6923076923076934</v>
+        <v>332.99492385786812</v>
       </c>
     </row>
   </sheetData>
@@ -2110,72 +2106,72 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>86</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B2">
         <v>10</v>
       </c>
       <c r="C2">
-        <v>3403.9</v>
+        <v>3124.8</v>
       </c>
       <c r="D2">
-        <v>2450.8000000000002</v>
+        <v>2418.9</v>
       </c>
       <c r="E2">
-        <v>2087.5555555555561</v>
+        <v>2675.666666666667</v>
       </c>
       <c r="F2">
-        <v>2602.333333333333</v>
+        <v>2806.1111111111109</v>
       </c>
       <c r="G2">
-        <v>3355.7</v>
+        <v>2847.3</v>
       </c>
       <c r="H2">
-        <v>2095.25</v>
+        <v>2675.666666666667</v>
       </c>
       <c r="I2">
-        <v>3293.7</v>
+        <v>2786</v>
       </c>
       <c r="J2">
-        <v>1349.7365875244141</v>
+        <v>1631.8635363578801</v>
       </c>
       <c r="K2">
-        <v>37.087136317277782</v>
+        <v>20.93520580812514</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mejoa del GAP al 9% pero destrucción de rutas buenas en anterior entrenamiento
</commit_message>
<xml_diff>
--- a/DRL_Routing_Summary_stochastic_sigma10%_AM.xlsx
+++ b/DRL_Routing_Summary_stochastic_sigma10%_AM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a9faf7a5fe1343c6/Desktop/Maestria/Tesis MSc/RoutingModel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="11_8B418FE71B54906DBDD3C5B532358AD3C21C4A92" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{41281C83-72D8-42E5-9F56-9A25540FB4C2}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_8B418FE7B124DC44BBA978B73C358AD3C21C4ABC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3B5F9EA6-FFCE-4181-AB76-D1AF3BFB7EE5}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -152,7 +152,7 @@
     <t>HGA-LNS Gap (%)</t>
   </si>
   <si>
-    <t>[0, 6, 7, 1, 0]</t>
+    <t>[0, 1, 7, 0]</t>
   </si>
   <si>
     <t>Optimal</t>
@@ -164,7 +164,7 @@
     <t>[0, 2, 1, 0]</t>
   </si>
   <si>
-    <t>[1, 0, 6, 7, 1]</t>
+    <t>[1, 8, 7, 6, 1]</t>
   </si>
   <si>
     <t>[1, 0, 2, 8, 1]</t>
@@ -191,19 +191,19 @@
     <t>[3, 5, 4, 3]</t>
   </si>
   <si>
-    <t>[4, 2, 4]</t>
+    <t>[4, 2, 8, 4]</t>
   </si>
   <si>
     <t>[4, 8, 2, 4]</t>
   </si>
   <si>
-    <t>[5, 3, 5]</t>
+    <t>[5, 3, 4, 5]</t>
   </si>
   <si>
     <t>[5, 4, 3, 5]</t>
   </si>
   <si>
-    <t>[6, 0, 1, 7, 6]</t>
+    <t>[6, 0, 7, 6]</t>
   </si>
   <si>
     <t>[6, 2, 8, 1, 6]</t>
@@ -212,13 +212,13 @@
     <t>[6, 2, 1, 6]</t>
   </si>
   <si>
-    <t>[7, 6, 2, 7]</t>
+    <t>[7, 1, 0, 6, 7]</t>
   </si>
   <si>
     <t>[7, 2, 6, 7]</t>
   </si>
   <si>
-    <t>[8, 0, 6, 8]</t>
+    <t>[8, 0, 1, 2, 8]</t>
   </si>
   <si>
     <t>[8, 2, 1, 0, 8]</t>
@@ -303,6 +303,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -650,19 +651,9 @@
   <dimension ref="A1:AQ11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="15.44140625" customWidth="1"/>
-    <col min="11" max="11" width="14.44140625" customWidth="1"/>
-    <col min="15" max="15" width="15.44140625" customWidth="1"/>
-    <col min="19" max="19" width="15.5546875" customWidth="1"/>
-    <col min="24" max="24" width="15.6640625" customWidth="1"/>
-    <col min="29" max="29" width="15.33203125" customWidth="1"/>
-    <col min="34" max="34" width="14" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="17.5546875" customWidth="1"/>
-    <col min="39" max="39" width="18.44140625" customWidth="1"/>
-    <col min="40" max="40" width="15.109375" customWidth="1"/>
-    <col min="41" max="41" width="15" customWidth="1"/>
-    <col min="42" max="42" width="16.33203125" customWidth="1"/>
-    <col min="43" max="43" width="19" customWidth="1"/>
+    <col min="3" max="3" width="19" customWidth="1"/>
+    <col min="12" max="12" width="12.21875" customWidth="1"/>
+    <col min="39" max="39" width="14.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:43" x14ac:dyDescent="0.3">
@@ -807,19 +798,19 @@
         <v>43</v>
       </c>
       <c r="D2">
-        <v>2403</v>
+        <v>2793</v>
       </c>
       <c r="E2">
-        <v>74.09</v>
+        <v>69.5</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
       </c>
       <c r="G2">
-        <v>2360.242422582282</v>
+        <v>2755.9708517519762</v>
       </c>
       <c r="H2">
-        <v>440.6687375381195</v>
+        <v>381.63032136162872</v>
       </c>
       <c r="I2">
         <v>100</v>
@@ -909,7 +900,7 @@
         <v>1</v>
       </c>
       <c r="AL2">
-        <v>29.818925233644858</v>
+        <v>18.428738317757009</v>
       </c>
       <c r="AM2">
         <v>4.3516355140186924</v>
@@ -938,16 +929,16 @@
         <v>47</v>
       </c>
       <c r="D3">
-        <v>3284</v>
+        <v>3987</v>
       </c>
       <c r="E3">
-        <v>74.09</v>
+        <v>73.150000000000006</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
       </c>
       <c r="G3">
-        <v>3416.1097767738888</v>
+        <v>4119.1097767738884</v>
       </c>
       <c r="H3">
         <v>430.07934961368261</v>
@@ -1040,7 +1031,7 @@
         <v>1</v>
       </c>
       <c r="AL3">
-        <v>28.60869565217391</v>
+        <v>13.32608695652174</v>
       </c>
       <c r="AM3">
         <v>63.891304347826093</v>
@@ -1331,19 +1322,19 @@
         <v>56</v>
       </c>
       <c r="D6">
-        <v>2006</v>
+        <v>2487</v>
       </c>
       <c r="E6">
-        <v>55.8</v>
+        <v>72.3</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
       </c>
       <c r="G6">
-        <v>1988.8867739611539</v>
+        <v>2466.0406641759591</v>
       </c>
       <c r="H6">
-        <v>248.96790977144721</v>
+        <v>304.92217063366388</v>
       </c>
       <c r="I6">
         <v>100</v>
@@ -1433,7 +1424,7 @@
         <v>1</v>
       </c>
       <c r="AL6">
-        <v>19.340570969039</v>
+        <v>0</v>
       </c>
       <c r="AM6">
         <v>0</v>
@@ -1462,19 +1453,19 @@
         <v>58</v>
       </c>
       <c r="D7">
-        <v>1008</v>
+        <v>2183</v>
       </c>
       <c r="E7">
-        <v>34.239999999999988</v>
+        <v>54.16</v>
       </c>
       <c r="F7" t="b">
         <v>1</v>
       </c>
       <c r="G7">
-        <v>1026.6930563382371</v>
+        <v>2205.8942248808889</v>
       </c>
       <c r="H7">
-        <v>292.34118593450211</v>
+        <v>358.04336816981629</v>
       </c>
       <c r="I7">
         <v>100</v>
@@ -1564,7 +1555,7 @@
         <v>1</v>
       </c>
       <c r="AL7">
-        <v>53.825011452130099</v>
+        <v>0</v>
       </c>
       <c r="AM7">
         <v>0</v>
@@ -1593,19 +1584,19 @@
         <v>60</v>
       </c>
       <c r="D8">
-        <v>3449</v>
+        <v>2419</v>
       </c>
       <c r="E8">
-        <v>74.59</v>
+        <v>58.06</v>
       </c>
       <c r="F8" t="b">
         <v>1</v>
       </c>
       <c r="G8">
-        <v>3443.7589494943331</v>
+        <v>2414.4611171195752</v>
       </c>
       <c r="H8">
-        <v>391.10814814573399</v>
+        <v>338.70959192129328</v>
       </c>
       <c r="I8">
         <v>100</v>
@@ -1695,7 +1686,7 @@
         <v>1</v>
       </c>
       <c r="AL8">
-        <v>28.769103676166871</v>
+        <v>50.04130524576621</v>
       </c>
       <c r="AM8">
         <v>3.1185460553490292</v>
@@ -1724,19 +1715,19 @@
         <v>63</v>
       </c>
       <c r="D9">
-        <v>3681</v>
+        <v>3378</v>
       </c>
       <c r="E9">
-        <v>66.430000000000007</v>
+        <v>74.09</v>
       </c>
       <c r="F9" t="b">
         <v>1</v>
       </c>
       <c r="G9">
-        <v>3676.3394265887018</v>
+        <v>3372.6184333728188</v>
       </c>
       <c r="H9">
-        <v>367.94400640819322</v>
+        <v>424.86514229295938</v>
       </c>
       <c r="I9">
         <v>100</v>
@@ -1826,7 +1817,7 @@
         <v>1</v>
       </c>
       <c r="AL9">
-        <v>0</v>
+        <v>8.2314588427057878</v>
       </c>
       <c r="AM9">
         <v>0</v>
@@ -1855,19 +1846,19 @@
         <v>65</v>
       </c>
       <c r="D10">
-        <v>1742</v>
+        <v>3415</v>
       </c>
       <c r="E10">
-        <v>63.13000000000001</v>
+        <v>75.17</v>
       </c>
       <c r="F10" t="b">
         <v>1</v>
       </c>
       <c r="G10">
-        <v>1770.757128269227</v>
+        <v>3448.205871494717</v>
       </c>
       <c r="H10">
-        <v>363.11846402797357</v>
+        <v>419.29308590854788</v>
       </c>
       <c r="I10">
         <v>100</v>
@@ -1957,7 +1948,7 @@
         <v>1</v>
       </c>
       <c r="AL10">
-        <v>48.989751098096633</v>
+        <v>0</v>
       </c>
       <c r="AM10">
         <v>30.21961932650073</v>
@@ -2150,7 +2141,7 @@
         <v>3124.8</v>
       </c>
       <c r="D2">
-        <v>2418.9</v>
+        <v>2727.8</v>
       </c>
       <c r="E2">
         <v>2675.666666666667</v>
@@ -2168,10 +2159,10 @@
         <v>2786</v>
       </c>
       <c r="J2">
-        <v>1631.8635363578801</v>
+        <v>881.74267435073853</v>
       </c>
       <c r="K2">
-        <v>20.93520580812514</v>
+        <v>9.0027589362750753</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Versión estable con 8.7% GAP
</commit_message>
<xml_diff>
--- a/DRL_Routing_Summary_stochastic_sigma10%_AM.xlsx
+++ b/DRL_Routing_Summary_stochastic_sigma10%_AM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a9faf7a5fe1343c6/Desktop/Maestria/Tesis MSc/RoutingModel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_8B418FE7B124DC44BBA978B73C358AD3C21C4ABC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3B5F9EA6-FFCE-4181-AB76-D1AF3BFB7EE5}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="11_8B418FE7368C1531740899143A358AD3C21C4B49" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A928560-A151-4C0A-A735-5B574C8EDA3E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,20 @@
     <sheet name="Per Node Results" sheetId="1" r:id="rId1"/>
     <sheet name="Summary" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -152,7 +165,7 @@
     <t>HGA-LNS Gap (%)</t>
   </si>
   <si>
-    <t>[0, 1, 7, 0]</t>
+    <t>[0, 6, 7, 1, 0]</t>
   </si>
   <si>
     <t>Optimal</t>
@@ -164,7 +177,7 @@
     <t>[0, 2, 1, 0]</t>
   </si>
   <si>
-    <t>[1, 8, 7, 6, 1]</t>
+    <t>[1, 0, 6, 7, 1]</t>
   </si>
   <si>
     <t>[1, 0, 2, 8, 1]</t>
@@ -203,7 +216,7 @@
     <t>[5, 4, 3, 5]</t>
   </si>
   <si>
-    <t>[6, 0, 7, 6]</t>
+    <t>[6, 0, 1, 7, 6]</t>
   </si>
   <si>
     <t>[6, 2, 8, 1, 6]</t>
@@ -212,7 +225,7 @@
     <t>[6, 2, 1, 6]</t>
   </si>
   <si>
-    <t>[7, 1, 0, 6, 7]</t>
+    <t>[7, 6, 2, 7]</t>
   </si>
   <si>
     <t>[7, 2, 6, 7]</t>
@@ -648,12 +661,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AQ11"/>
+  <dimension ref="A1:AQ13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="12" max="12" width="12.21875" customWidth="1"/>
-    <col min="39" max="39" width="14.109375" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" customWidth="1"/>
+    <col min="38" max="38" width="15.5546875" customWidth="1"/>
+    <col min="39" max="39" width="19.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:43" x14ac:dyDescent="0.3">
@@ -798,19 +811,19 @@
         <v>43</v>
       </c>
       <c r="D2">
-        <v>2793</v>
+        <v>2403</v>
       </c>
       <c r="E2">
-        <v>69.5</v>
+        <v>74.09</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
       </c>
       <c r="G2">
-        <v>2755.9708517519762</v>
+        <v>2360.242422582282</v>
       </c>
       <c r="H2">
-        <v>381.63032136162872</v>
+        <v>440.6687375381195</v>
       </c>
       <c r="I2">
         <v>100</v>
@@ -900,7 +913,7 @@
         <v>1</v>
       </c>
       <c r="AL2">
-        <v>18.428738317757009</v>
+        <v>29.818925233644858</v>
       </c>
       <c r="AM2">
         <v>4.3516355140186924</v>
@@ -929,16 +942,16 @@
         <v>47</v>
       </c>
       <c r="D3">
-        <v>3987</v>
+        <v>3284</v>
       </c>
       <c r="E3">
-        <v>73.150000000000006</v>
+        <v>74.09</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
       </c>
       <c r="G3">
-        <v>4119.1097767738884</v>
+        <v>3416.1097767738888</v>
       </c>
       <c r="H3">
         <v>430.07934961368261</v>
@@ -1031,7 +1044,7 @@
         <v>1</v>
       </c>
       <c r="AL3">
-        <v>13.32608695652174</v>
+        <v>28.60869565217391</v>
       </c>
       <c r="AM3">
         <v>63.891304347826093</v>
@@ -1584,19 +1597,19 @@
         <v>60</v>
       </c>
       <c r="D8">
-        <v>2419</v>
+        <v>3449</v>
       </c>
       <c r="E8">
-        <v>58.06</v>
+        <v>74.59</v>
       </c>
       <c r="F8" t="b">
         <v>1</v>
       </c>
       <c r="G8">
-        <v>2414.4611171195752</v>
+        <v>3443.7589494943331</v>
       </c>
       <c r="H8">
-        <v>338.70959192129328</v>
+        <v>391.10814814573399</v>
       </c>
       <c r="I8">
         <v>100</v>
@@ -1686,7 +1699,7 @@
         <v>1</v>
       </c>
       <c r="AL8">
-        <v>50.04130524576621</v>
+        <v>28.769103676166871</v>
       </c>
       <c r="AM8">
         <v>3.1185460553490292</v>
@@ -1715,19 +1728,19 @@
         <v>63</v>
       </c>
       <c r="D9">
-        <v>3378</v>
+        <v>3681</v>
       </c>
       <c r="E9">
-        <v>74.09</v>
+        <v>66.430000000000007</v>
       </c>
       <c r="F9" t="b">
         <v>1</v>
       </c>
       <c r="G9">
-        <v>3372.6184333728188</v>
+        <v>3676.3394265887018</v>
       </c>
       <c r="H9">
-        <v>424.86514229295938</v>
+        <v>367.94400640819322</v>
       </c>
       <c r="I9">
         <v>100</v>
@@ -1817,7 +1830,7 @@
         <v>1</v>
       </c>
       <c r="AL9">
-        <v>8.2314588427057878</v>
+        <v>0</v>
       </c>
       <c r="AM9">
         <v>0</v>
@@ -2083,6 +2096,32 @@
       </c>
       <c r="AQ11">
         <v>332.99492385786812</v>
+      </c>
+    </row>
+    <row r="13" spans="1:43" x14ac:dyDescent="0.3">
+      <c r="AL13">
+        <f>AVERAGE(AL2:AL11)</f>
+        <v>8.7196724561985626</v>
+      </c>
+      <c r="AM13">
+        <f t="shared" ref="AM13:AQ13" si="0">AVERAGE(AM2:AM11)</f>
+        <v>17.228499827235012</v>
+      </c>
+      <c r="AN13">
+        <f t="shared" si="0"/>
+        <v>13.554816077132825</v>
+      </c>
+      <c r="AO13">
+        <f t="shared" si="0"/>
+        <v>33.611346991321717</v>
+      </c>
+      <c r="AP13">
+        <f t="shared" si="0"/>
+        <v>17.228499827235012</v>
+      </c>
+      <c r="AQ13">
+        <f t="shared" si="0"/>
+        <v>34.943955686973894</v>
       </c>
     </row>
   </sheetData>
@@ -2141,7 +2180,7 @@
         <v>3124.8</v>
       </c>
       <c r="D2">
-        <v>2727.8</v>
+        <v>2751.8</v>
       </c>
       <c r="E2">
         <v>2675.666666666667</v>
@@ -2159,10 +2198,10 @@
         <v>2786</v>
       </c>
       <c r="J2">
-        <v>881.74267435073853</v>
+        <v>951.65280675888062</v>
       </c>
       <c r="K2">
-        <v>9.0027589362750753</v>
+        <v>8.7196724561985643</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Version con 5.4% de GAP
</commit_message>
<xml_diff>
--- a/DRL_Routing_Summary_stochastic_sigma10%_AM.xlsx
+++ b/DRL_Routing_Summary_stochastic_sigma10%_AM.xlsx
@@ -808,20 +808,20 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>[1, 0, 6, 7, 1]</t>
+          <t>[1, 8, 7, 6, 1]</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3284</v>
+        <v>3987</v>
       </c>
       <c r="E3" t="n">
-        <v>74.09</v>
+        <v>73.15000000000001</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>3416.109776773889</v>
+        <v>4119.109776773888</v>
       </c>
       <c r="H3" t="n">
         <v>430.0793496136826</v>
@@ -934,7 +934,7 @@
         <v>1</v>
       </c>
       <c r="AL3" t="n">
-        <v>28.60869565217391</v>
+        <v>13.32608695652174</v>
       </c>
       <c r="AM3" t="n">
         <v>63.89130434782609</v>
@@ -2258,7 +2258,7 @@
         <v>3124.8</v>
       </c>
       <c r="D2" t="n">
-        <v>2819.4</v>
+        <v>2889.7</v>
       </c>
       <c r="E2" t="n">
         <v>2675.666666666667</v>
@@ -2276,10 +2276,10 @@
         <v>2786</v>
       </c>
       <c r="J2" t="n">
-        <v>812.9796824455261</v>
+        <v>1057.672137498856</v>
       </c>
       <c r="K2" t="n">
-        <v>6.989988750152944</v>
+        <v>5.461727880587726</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Baseline AM-PPO independiente con 0.93% GAP en 10 nodos
</commit_message>
<xml_diff>
--- a/DRL_Routing_Summary_stochastic_sigma10%_AM.xlsx
+++ b/DRL_Routing_Summary_stochastic_sigma10%_AM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a9faf7a5fe1343c6/Desktop/Maestria/Tesis MSc/RoutingModel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_8B418FE7E5B4918DE99A2E9632358AD3C21C551D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3D86A6C5-8E82-4434-8F24-38D3F886DA68}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_8B418FE74184D7CD6152BD7723358AD3C21C4A99" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5058B4F7-75CB-4410-AC94-4BE6164AD104}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="75">
   <si>
     <t>Start Node</t>
   </si>
@@ -152,6 +152,9 @@
     <t>HGA-LNS Gap (%)</t>
   </si>
   <si>
+    <t>DRL Stoch Gap (%)</t>
+  </si>
+  <si>
     <t>[0, 6, 0]</t>
   </si>
   <si>
@@ -237,6 +240,9 @@
   </si>
   <si>
     <t>DRL Avg Gap (%)</t>
+  </si>
+  <si>
+    <t>DRL Avg Stoch Gap (%)</t>
   </si>
   <si>
     <t>AM</t>
@@ -602,13 +608,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AQ11"/>
+  <dimension ref="A1:AR11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="13" max="13" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="12" customWidth="1"/>
+    <col min="44" max="44" width="17.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -738,8 +745,11 @@
       <c r="AQ1" s="1" t="s">
         <v>42</v>
       </c>
+      <c r="AR1" s="1" t="s">
+        <v>43</v>
+      </c>
     </row>
-    <row r="2" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>0</v>
       </c>
@@ -747,7 +757,7 @@
         <v>51</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D2">
         <v>1700</v>
@@ -759,19 +769,19 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>1669.7658270608231</v>
+        <v>1678.621211291141</v>
       </c>
       <c r="H2">
-        <v>311.59985257011931</v>
+        <v>220.33436876905969</v>
       </c>
       <c r="I2">
         <v>100</v>
       </c>
       <c r="J2" t="s">
+        <v>45</v>
+      </c>
+      <c r="K2" t="s">
         <v>44</v>
-      </c>
-      <c r="K2" t="s">
-        <v>43</v>
       </c>
       <c r="L2">
         <v>1700</v>
@@ -783,7 +793,7 @@
         <v>1</v>
       </c>
       <c r="O2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="P2">
         <v>1700</v>
@@ -795,7 +805,7 @@
         <v>1</v>
       </c>
       <c r="S2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="T2">
         <v>1700</v>
@@ -807,10 +817,10 @@
         <v>1</v>
       </c>
       <c r="W2" t="s">
+        <v>45</v>
+      </c>
+      <c r="X2" t="s">
         <v>44</v>
-      </c>
-      <c r="X2" t="s">
-        <v>43</v>
       </c>
       <c r="Y2">
         <v>1700</v>
@@ -822,10 +832,10 @@
         <v>1</v>
       </c>
       <c r="AB2" t="s">
+        <v>45</v>
+      </c>
+      <c r="AC2" t="s">
         <v>44</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>43</v>
       </c>
       <c r="AD2">
         <v>1700</v>
@@ -837,10 +847,10 @@
         <v>1</v>
       </c>
       <c r="AG2" t="s">
+        <v>45</v>
+      </c>
+      <c r="AH2" t="s">
         <v>44</v>
-      </c>
-      <c r="AH2" t="s">
-        <v>43</v>
       </c>
       <c r="AI2">
         <v>1700</v>
@@ -869,8 +879,11 @@
       <c r="AQ2">
         <v>0</v>
       </c>
+      <c r="AR2">
+        <v>1.2575758064034721</v>
+      </c>
     </row>
-    <row r="3" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -878,7 +891,7 @@
         <v>78</v>
       </c>
       <c r="C3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D3">
         <v>1681</v>
@@ -890,19 +903,19 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>1671.810280950222</v>
+        <v>1675.694313232834</v>
       </c>
       <c r="H3">
-        <v>336.36853380500128</v>
+        <v>194.20246353923719</v>
       </c>
       <c r="I3">
         <v>100</v>
       </c>
       <c r="J3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="L3">
         <v>1854</v>
@@ -914,7 +927,7 @@
         <v>1</v>
       </c>
       <c r="O3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="P3">
         <v>1403</v>
@@ -926,7 +939,7 @@
         <v>1</v>
       </c>
       <c r="S3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="T3">
         <v>1681</v>
@@ -938,10 +951,10 @@
         <v>1</v>
       </c>
       <c r="W3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="X3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="Y3">
         <v>1854</v>
@@ -953,10 +966,10 @@
         <v>1</v>
       </c>
       <c r="AB3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="AD3">
         <v>1403</v>
@@ -968,10 +981,10 @@
         <v>1</v>
       </c>
       <c r="AG3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AH3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="AI3">
         <v>1854</v>
@@ -1000,8 +1013,11 @@
       <c r="AQ3">
         <v>0</v>
       </c>
+      <c r="AR3">
+        <v>9.6173509583153418</v>
+      </c>
     </row>
-    <row r="4" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
@@ -1009,7 +1025,7 @@
         <v>48</v>
       </c>
       <c r="C4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D4">
         <v>3406</v>
@@ -1021,19 +1037,19 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>3317.933175955613</v>
+        <v>3355.1545954312978</v>
       </c>
       <c r="H4">
-        <v>369.66655042283179</v>
+        <v>213.4270823970223</v>
       </c>
       <c r="I4">
         <v>100</v>
       </c>
       <c r="J4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="L4">
         <v>3406</v>
@@ -1045,7 +1061,7 @@
         <v>1</v>
       </c>
       <c r="O4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="P4">
         <v>919</v>
@@ -1057,7 +1073,7 @@
         <v>1</v>
       </c>
       <c r="S4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="T4">
         <v>3406</v>
@@ -1069,10 +1085,10 @@
         <v>1</v>
       </c>
       <c r="W4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="X4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Y4">
         <v>3406</v>
@@ -1084,10 +1100,10 @@
         <v>1</v>
       </c>
       <c r="AB4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AD4">
         <v>919</v>
@@ -1099,10 +1115,10 @@
         <v>1</v>
       </c>
       <c r="AG4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AH4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AI4">
         <v>3406</v>
@@ -1131,8 +1147,11 @@
       <c r="AQ4">
         <v>0</v>
       </c>
+      <c r="AR4">
+        <v>1.4928186896271931</v>
+      </c>
     </row>
-    <row r="5" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
@@ -1140,7 +1159,7 @@
         <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D5">
         <v>720</v>
@@ -1152,19 +1171,19 @@
         <v>1</v>
       </c>
       <c r="G5">
-        <v>695.41226230256564</v>
+        <v>702.61384394010815</v>
       </c>
       <c r="H5">
-        <v>331.99745614424558</v>
+        <v>234.7576525762795</v>
       </c>
       <c r="I5">
         <v>100</v>
       </c>
       <c r="J5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="L5">
         <v>720</v>
@@ -1176,7 +1195,7 @@
         <v>1</v>
       </c>
       <c r="O5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="P5">
         <v>720</v>
@@ -1188,7 +1207,7 @@
         <v>1</v>
       </c>
       <c r="S5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="T5">
         <v>720</v>
@@ -1200,10 +1219,10 @@
         <v>1</v>
       </c>
       <c r="W5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="X5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Y5">
         <v>720</v>
@@ -1215,10 +1234,10 @@
         <v>1</v>
       </c>
       <c r="AB5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="AD5">
         <v>720</v>
@@ -1230,10 +1249,10 @@
         <v>1</v>
       </c>
       <c r="AG5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AH5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="AI5">
         <v>720</v>
@@ -1262,8 +1281,11 @@
       <c r="AQ5">
         <v>0</v>
       </c>
+      <c r="AR5">
+        <v>2.4147438972072011</v>
+      </c>
     </row>
-    <row r="6" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>4</v>
       </c>
@@ -1271,7 +1293,7 @@
         <v>89</v>
       </c>
       <c r="C6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D6">
         <v>923</v>
@@ -1283,19 +1305,19 @@
         <v>1</v>
       </c>
       <c r="G6">
-        <v>940.95393561404239</v>
+        <v>935.69534962167597</v>
       </c>
       <c r="H6">
-        <v>293.01785016507142</v>
+        <v>207.19490886042581</v>
       </c>
       <c r="I6">
         <v>100</v>
       </c>
       <c r="J6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="L6">
         <v>923</v>
@@ -1307,7 +1329,7 @@
         <v>1</v>
       </c>
       <c r="O6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="P6">
         <v>923</v>
@@ -1319,7 +1341,7 @@
         <v>1</v>
       </c>
       <c r="S6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="T6">
         <v>923</v>
@@ -1331,10 +1353,10 @@
         <v>1</v>
       </c>
       <c r="W6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="X6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Y6">
         <v>923</v>
@@ -1346,10 +1368,10 @@
         <v>1</v>
       </c>
       <c r="AB6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="AD6">
         <v>923</v>
@@ -1361,10 +1383,10 @@
         <v>1</v>
       </c>
       <c r="AG6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AH6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="AI6">
         <v>923</v>
@@ -1393,8 +1415,11 @@
       <c r="AQ6">
         <v>0</v>
       </c>
+      <c r="AR6">
+        <v>-1.3754441626951219</v>
+      </c>
     </row>
-    <row r="7" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>5</v>
       </c>
@@ -1402,7 +1427,7 @@
         <v>79</v>
       </c>
       <c r="C7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D7">
         <v>778</v>
@@ -1414,19 +1439,19 @@
         <v>1</v>
       </c>
       <c r="G7">
-        <v>816.15283011474969</v>
+        <v>804.97812489559783</v>
       </c>
       <c r="H7">
-        <v>285.12922831637229</v>
+        <v>201.61681085699419</v>
       </c>
       <c r="I7">
         <v>100</v>
       </c>
       <c r="J7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L7">
         <v>778</v>
@@ -1438,7 +1463,7 @@
         <v>1</v>
       </c>
       <c r="O7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="P7">
         <v>778</v>
@@ -1450,7 +1475,7 @@
         <v>1</v>
       </c>
       <c r="S7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="T7">
         <v>778</v>
@@ -1462,10 +1487,10 @@
         <v>1</v>
       </c>
       <c r="W7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="X7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="Y7">
         <v>778</v>
@@ -1477,10 +1502,10 @@
         <v>1</v>
       </c>
       <c r="AB7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="AD7">
         <v>778</v>
@@ -1492,10 +1517,10 @@
         <v>1</v>
       </c>
       <c r="AG7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AH7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="AI7">
         <v>778</v>
@@ -1524,8 +1549,11 @@
       <c r="AQ7">
         <v>0</v>
       </c>
+      <c r="AR7">
+        <v>-3.467625307917459</v>
+      </c>
     </row>
-    <row r="8" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>6</v>
       </c>
@@ -1533,7 +1561,7 @@
         <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D8">
         <v>629</v>
@@ -1545,19 +1573,19 @@
         <v>1</v>
       </c>
       <c r="G8">
-        <v>698.26518634668707</v>
+        <v>677.97788296589215</v>
       </c>
       <c r="H8">
-        <v>301.30338115965378</v>
+        <v>213.0536640124262</v>
       </c>
       <c r="I8">
         <v>100</v>
       </c>
       <c r="J8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K8" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="L8">
         <v>629</v>
@@ -1569,7 +1597,7 @@
         <v>1</v>
       </c>
       <c r="O8" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="P8">
         <v>-6</v>
@@ -1581,7 +1609,7 @@
         <v>1</v>
       </c>
       <c r="S8" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="T8">
         <v>-6</v>
@@ -1593,10 +1621,10 @@
         <v>1</v>
       </c>
       <c r="W8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="X8" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="Y8">
         <v>-6</v>
@@ -1608,10 +1636,10 @@
         <v>1</v>
       </c>
       <c r="AB8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC8" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="AD8">
         <v>-6</v>
@@ -1623,10 +1651,10 @@
         <v>1</v>
       </c>
       <c r="AG8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AH8" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="AI8">
         <v>-6</v>
@@ -1655,8 +1683,11 @@
       <c r="AQ8">
         <v>100.95389507154211</v>
       </c>
+      <c r="AR8">
+        <v>-7.7866268626219632</v>
+      </c>
     </row>
-    <row r="9" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>7</v>
       </c>
@@ -1664,7 +1695,7 @@
         <v>84</v>
       </c>
       <c r="C9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D9">
         <v>1609</v>
@@ -1676,19 +1707,19 @@
         <v>1</v>
       </c>
       <c r="G9">
-        <v>1565.1632116645701</v>
+        <v>1578.0027097025779</v>
       </c>
       <c r="H9">
-        <v>294.19109435479822</v>
+        <v>208.02451778296921</v>
       </c>
       <c r="I9">
         <v>100</v>
       </c>
       <c r="J9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="L9">
         <v>1609</v>
@@ -1700,7 +1731,7 @@
         <v>1</v>
       </c>
       <c r="O9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="P9">
         <v>40</v>
@@ -1712,7 +1743,7 @@
         <v>1</v>
       </c>
       <c r="S9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="T9">
         <v>40</v>
@@ -1724,10 +1755,10 @@
         <v>1</v>
       </c>
       <c r="W9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="X9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Y9">
         <v>40</v>
@@ -1739,10 +1770,10 @@
         <v>1</v>
       </c>
       <c r="AB9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="AD9">
         <v>40</v>
@@ -1754,10 +1785,10 @@
         <v>1</v>
       </c>
       <c r="AG9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AH9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="AI9">
         <v>40</v>
@@ -1786,8 +1817,11 @@
       <c r="AQ9">
         <v>97.513983840894966</v>
       </c>
+      <c r="AR9">
+        <v>1.9264941141965239</v>
+      </c>
     </row>
-    <row r="10" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>8</v>
       </c>
@@ -1795,7 +1829,7 @@
         <v>57</v>
       </c>
       <c r="C10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D10">
         <v>3357</v>
@@ -1807,19 +1841,19 @@
         <v>1</v>
       </c>
       <c r="G10">
-        <v>3325.0942811978439</v>
+        <v>3338.5792246608871</v>
       </c>
       <c r="H10">
-        <v>375.71286905536999</v>
+        <v>216.9179260871245</v>
       </c>
       <c r="I10">
         <v>100</v>
       </c>
       <c r="J10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="L10">
         <v>3357</v>
@@ -1831,7 +1865,7 @@
         <v>1</v>
       </c>
       <c r="O10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="P10">
         <v>3357</v>
@@ -1843,7 +1877,7 @@
         <v>1</v>
       </c>
       <c r="S10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="T10">
         <v>3357</v>
@@ -1855,10 +1889,10 @@
         <v>1</v>
       </c>
       <c r="W10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="X10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Y10">
         <v>3357</v>
@@ -1870,10 +1904,10 @@
         <v>1</v>
       </c>
       <c r="AB10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="AD10">
         <v>3357</v>
@@ -1885,10 +1919,10 @@
         <v>1</v>
       </c>
       <c r="AG10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AH10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="AI10">
         <v>3357</v>
@@ -1917,8 +1951,11 @@
       <c r="AQ10">
         <v>0</v>
       </c>
+      <c r="AR10">
+        <v>0.54872729636917883</v>
+      </c>
     </row>
-    <row r="11" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>9</v>
       </c>
@@ -1926,7 +1963,7 @@
         <v>78</v>
       </c>
       <c r="C11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D11">
         <v>-4028</v>
@@ -1938,19 +1975,19 @@
         <v>1</v>
       </c>
       <c r="G11">
-        <v>-4029.4891397464248</v>
+        <v>-4029.0529808128308</v>
       </c>
       <c r="H11">
-        <v>273.57539912817651</v>
+        <v>193.44701988934989</v>
       </c>
       <c r="I11">
         <v>100</v>
       </c>
       <c r="J11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L11">
         <v>-4028</v>
@@ -1962,7 +1999,7 @@
         <v>1</v>
       </c>
       <c r="O11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="P11">
         <v>-4028</v>
@@ -1974,7 +2011,7 @@
         <v>1</v>
       </c>
       <c r="S11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="T11">
         <v>-4028</v>
@@ -1986,10 +2023,10 @@
         <v>1</v>
       </c>
       <c r="W11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="X11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="Y11">
         <v>-4028</v>
@@ -2001,10 +2038,10 @@
         <v>1</v>
       </c>
       <c r="AB11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="AD11">
         <v>-4028</v>
@@ -2016,10 +2053,10 @@
         <v>1</v>
       </c>
       <c r="AG11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AH11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="AI11">
         <v>-4028</v>
@@ -2047,6 +2084,9 @@
       </c>
       <c r="AQ11">
         <v>0</v>
+      </c>
+      <c r="AR11">
+        <v>2.614152961348722E-2</v>
       </c>
     </row>
   </sheetData>
@@ -2056,47 +2096,50 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B2">
         <v>10</v>
@@ -2123,10 +2166,13 @@
         <v>874.4</v>
       </c>
       <c r="J2">
-        <v>1206.2921981811519</v>
+        <v>1267.504115819931</v>
       </c>
       <c r="K2">
         <v>0.93311758360302055</v>
+      </c>
+      <c r="L2">
+        <v>0.46541559584978531</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Baseline PPO-AM independiente con 0.93% de GAP
</commit_message>
<xml_diff>
--- a/DRL_Routing_Summary_stochastic_sigma10%_AM.xlsx
+++ b/DRL_Routing_Summary_stochastic_sigma10%_AM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a9faf7a5fe1343c6/Desktop/Maestria/Tesis MSc/RoutingModel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_8B418FE7E5B4918DE99A2E9632358AD3C21C551D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3D86A6C5-8E82-4434-8F24-38D3F886DA68}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_8B418FE74184D7CD6152BD7723358AD3C21C4A99" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5058B4F7-75CB-4410-AC94-4BE6164AD104}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="75">
   <si>
     <t>Start Node</t>
   </si>
@@ -152,6 +152,9 @@
     <t>HGA-LNS Gap (%)</t>
   </si>
   <si>
+    <t>DRL Stoch Gap (%)</t>
+  </si>
+  <si>
     <t>[0, 6, 0]</t>
   </si>
   <si>
@@ -237,6 +240,9 @@
   </si>
   <si>
     <t>DRL Avg Gap (%)</t>
+  </si>
+  <si>
+    <t>DRL Avg Stoch Gap (%)</t>
   </si>
   <si>
     <t>AM</t>
@@ -602,13 +608,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AQ11"/>
+  <dimension ref="A1:AR11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="13" max="13" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="12" customWidth="1"/>
+    <col min="44" max="44" width="17.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -738,8 +745,11 @@
       <c r="AQ1" s="1" t="s">
         <v>42</v>
       </c>
+      <c r="AR1" s="1" t="s">
+        <v>43</v>
+      </c>
     </row>
-    <row r="2" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>0</v>
       </c>
@@ -747,7 +757,7 @@
         <v>51</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D2">
         <v>1700</v>
@@ -759,19 +769,19 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>1669.7658270608231</v>
+        <v>1678.621211291141</v>
       </c>
       <c r="H2">
-        <v>311.59985257011931</v>
+        <v>220.33436876905969</v>
       </c>
       <c r="I2">
         <v>100</v>
       </c>
       <c r="J2" t="s">
+        <v>45</v>
+      </c>
+      <c r="K2" t="s">
         <v>44</v>
-      </c>
-      <c r="K2" t="s">
-        <v>43</v>
       </c>
       <c r="L2">
         <v>1700</v>
@@ -783,7 +793,7 @@
         <v>1</v>
       </c>
       <c r="O2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="P2">
         <v>1700</v>
@@ -795,7 +805,7 @@
         <v>1</v>
       </c>
       <c r="S2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="T2">
         <v>1700</v>
@@ -807,10 +817,10 @@
         <v>1</v>
       </c>
       <c r="W2" t="s">
+        <v>45</v>
+      </c>
+      <c r="X2" t="s">
         <v>44</v>
-      </c>
-      <c r="X2" t="s">
-        <v>43</v>
       </c>
       <c r="Y2">
         <v>1700</v>
@@ -822,10 +832,10 @@
         <v>1</v>
       </c>
       <c r="AB2" t="s">
+        <v>45</v>
+      </c>
+      <c r="AC2" t="s">
         <v>44</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>43</v>
       </c>
       <c r="AD2">
         <v>1700</v>
@@ -837,10 +847,10 @@
         <v>1</v>
       </c>
       <c r="AG2" t="s">
+        <v>45</v>
+      </c>
+      <c r="AH2" t="s">
         <v>44</v>
-      </c>
-      <c r="AH2" t="s">
-        <v>43</v>
       </c>
       <c r="AI2">
         <v>1700</v>
@@ -869,8 +879,11 @@
       <c r="AQ2">
         <v>0</v>
       </c>
+      <c r="AR2">
+        <v>1.2575758064034721</v>
+      </c>
     </row>
-    <row r="3" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -878,7 +891,7 @@
         <v>78</v>
       </c>
       <c r="C3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D3">
         <v>1681</v>
@@ -890,19 +903,19 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>1671.810280950222</v>
+        <v>1675.694313232834</v>
       </c>
       <c r="H3">
-        <v>336.36853380500128</v>
+        <v>194.20246353923719</v>
       </c>
       <c r="I3">
         <v>100</v>
       </c>
       <c r="J3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="L3">
         <v>1854</v>
@@ -914,7 +927,7 @@
         <v>1</v>
       </c>
       <c r="O3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="P3">
         <v>1403</v>
@@ -926,7 +939,7 @@
         <v>1</v>
       </c>
       <c r="S3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="T3">
         <v>1681</v>
@@ -938,10 +951,10 @@
         <v>1</v>
       </c>
       <c r="W3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="X3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="Y3">
         <v>1854</v>
@@ -953,10 +966,10 @@
         <v>1</v>
       </c>
       <c r="AB3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="AD3">
         <v>1403</v>
@@ -968,10 +981,10 @@
         <v>1</v>
       </c>
       <c r="AG3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AH3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="AI3">
         <v>1854</v>
@@ -1000,8 +1013,11 @@
       <c r="AQ3">
         <v>0</v>
       </c>
+      <c r="AR3">
+        <v>9.6173509583153418</v>
+      </c>
     </row>
-    <row r="4" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
@@ -1009,7 +1025,7 @@
         <v>48</v>
       </c>
       <c r="C4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D4">
         <v>3406</v>
@@ -1021,19 +1037,19 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>3317.933175955613</v>
+        <v>3355.1545954312978</v>
       </c>
       <c r="H4">
-        <v>369.66655042283179</v>
+        <v>213.4270823970223</v>
       </c>
       <c r="I4">
         <v>100</v>
       </c>
       <c r="J4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="L4">
         <v>3406</v>
@@ -1045,7 +1061,7 @@
         <v>1</v>
       </c>
       <c r="O4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="P4">
         <v>919</v>
@@ -1057,7 +1073,7 @@
         <v>1</v>
       </c>
       <c r="S4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="T4">
         <v>3406</v>
@@ -1069,10 +1085,10 @@
         <v>1</v>
       </c>
       <c r="W4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="X4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="Y4">
         <v>3406</v>
@@ -1084,10 +1100,10 @@
         <v>1</v>
       </c>
       <c r="AB4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AD4">
         <v>919</v>
@@ -1099,10 +1115,10 @@
         <v>1</v>
       </c>
       <c r="AG4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AH4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AI4">
         <v>3406</v>
@@ -1131,8 +1147,11 @@
       <c r="AQ4">
         <v>0</v>
       </c>
+      <c r="AR4">
+        <v>1.4928186896271931</v>
+      </c>
     </row>
-    <row r="5" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
@@ -1140,7 +1159,7 @@
         <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D5">
         <v>720</v>
@@ -1152,19 +1171,19 @@
         <v>1</v>
       </c>
       <c r="G5">
-        <v>695.41226230256564</v>
+        <v>702.61384394010815</v>
       </c>
       <c r="H5">
-        <v>331.99745614424558</v>
+        <v>234.7576525762795</v>
       </c>
       <c r="I5">
         <v>100</v>
       </c>
       <c r="J5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="L5">
         <v>720</v>
@@ -1176,7 +1195,7 @@
         <v>1</v>
       </c>
       <c r="O5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="P5">
         <v>720</v>
@@ -1188,7 +1207,7 @@
         <v>1</v>
       </c>
       <c r="S5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="T5">
         <v>720</v>
@@ -1200,10 +1219,10 @@
         <v>1</v>
       </c>
       <c r="W5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="X5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Y5">
         <v>720</v>
@@ -1215,10 +1234,10 @@
         <v>1</v>
       </c>
       <c r="AB5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="AD5">
         <v>720</v>
@@ -1230,10 +1249,10 @@
         <v>1</v>
       </c>
       <c r="AG5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AH5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="AI5">
         <v>720</v>
@@ -1262,8 +1281,11 @@
       <c r="AQ5">
         <v>0</v>
       </c>
+      <c r="AR5">
+        <v>2.4147438972072011</v>
+      </c>
     </row>
-    <row r="6" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>4</v>
       </c>
@@ -1271,7 +1293,7 @@
         <v>89</v>
       </c>
       <c r="C6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D6">
         <v>923</v>
@@ -1283,19 +1305,19 @@
         <v>1</v>
       </c>
       <c r="G6">
-        <v>940.95393561404239</v>
+        <v>935.69534962167597</v>
       </c>
       <c r="H6">
-        <v>293.01785016507142</v>
+        <v>207.19490886042581</v>
       </c>
       <c r="I6">
         <v>100</v>
       </c>
       <c r="J6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="L6">
         <v>923</v>
@@ -1307,7 +1329,7 @@
         <v>1</v>
       </c>
       <c r="O6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="P6">
         <v>923</v>
@@ -1319,7 +1341,7 @@
         <v>1</v>
       </c>
       <c r="S6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="T6">
         <v>923</v>
@@ -1331,10 +1353,10 @@
         <v>1</v>
       </c>
       <c r="W6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="X6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Y6">
         <v>923</v>
@@ -1346,10 +1368,10 @@
         <v>1</v>
       </c>
       <c r="AB6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="AD6">
         <v>923</v>
@@ -1361,10 +1383,10 @@
         <v>1</v>
       </c>
       <c r="AG6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AH6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="AI6">
         <v>923</v>
@@ -1393,8 +1415,11 @@
       <c r="AQ6">
         <v>0</v>
       </c>
+      <c r="AR6">
+        <v>-1.3754441626951219</v>
+      </c>
     </row>
-    <row r="7" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>5</v>
       </c>
@@ -1402,7 +1427,7 @@
         <v>79</v>
       </c>
       <c r="C7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D7">
         <v>778</v>
@@ -1414,19 +1439,19 @@
         <v>1</v>
       </c>
       <c r="G7">
-        <v>816.15283011474969</v>
+        <v>804.97812489559783</v>
       </c>
       <c r="H7">
-        <v>285.12922831637229</v>
+        <v>201.61681085699419</v>
       </c>
       <c r="I7">
         <v>100</v>
       </c>
       <c r="J7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L7">
         <v>778</v>
@@ -1438,7 +1463,7 @@
         <v>1</v>
       </c>
       <c r="O7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="P7">
         <v>778</v>
@@ -1450,7 +1475,7 @@
         <v>1</v>
       </c>
       <c r="S7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="T7">
         <v>778</v>
@@ -1462,10 +1487,10 @@
         <v>1</v>
       </c>
       <c r="W7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="X7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="Y7">
         <v>778</v>
@@ -1477,10 +1502,10 @@
         <v>1</v>
       </c>
       <c r="AB7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="AD7">
         <v>778</v>
@@ -1492,10 +1517,10 @@
         <v>1</v>
       </c>
       <c r="AG7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AH7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="AI7">
         <v>778</v>
@@ -1524,8 +1549,11 @@
       <c r="AQ7">
         <v>0</v>
       </c>
+      <c r="AR7">
+        <v>-3.467625307917459</v>
+      </c>
     </row>
-    <row r="8" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>6</v>
       </c>
@@ -1533,7 +1561,7 @@
         <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D8">
         <v>629</v>
@@ -1545,19 +1573,19 @@
         <v>1</v>
       </c>
       <c r="G8">
-        <v>698.26518634668707</v>
+        <v>677.97788296589215</v>
       </c>
       <c r="H8">
-        <v>301.30338115965378</v>
+        <v>213.0536640124262</v>
       </c>
       <c r="I8">
         <v>100</v>
       </c>
       <c r="J8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K8" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="L8">
         <v>629</v>
@@ -1569,7 +1597,7 @@
         <v>1</v>
       </c>
       <c r="O8" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="P8">
         <v>-6</v>
@@ -1581,7 +1609,7 @@
         <v>1</v>
       </c>
       <c r="S8" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="T8">
         <v>-6</v>
@@ -1593,10 +1621,10 @@
         <v>1</v>
       </c>
       <c r="W8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="X8" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="Y8">
         <v>-6</v>
@@ -1608,10 +1636,10 @@
         <v>1</v>
       </c>
       <c r="AB8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC8" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="AD8">
         <v>-6</v>
@@ -1623,10 +1651,10 @@
         <v>1</v>
       </c>
       <c r="AG8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AH8" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="AI8">
         <v>-6</v>
@@ -1655,8 +1683,11 @@
       <c r="AQ8">
         <v>100.95389507154211</v>
       </c>
+      <c r="AR8">
+        <v>-7.7866268626219632</v>
+      </c>
     </row>
-    <row r="9" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>7</v>
       </c>
@@ -1664,7 +1695,7 @@
         <v>84</v>
       </c>
       <c r="C9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D9">
         <v>1609</v>
@@ -1676,19 +1707,19 @@
         <v>1</v>
       </c>
       <c r="G9">
-        <v>1565.1632116645701</v>
+        <v>1578.0027097025779</v>
       </c>
       <c r="H9">
-        <v>294.19109435479822</v>
+        <v>208.02451778296921</v>
       </c>
       <c r="I9">
         <v>100</v>
       </c>
       <c r="J9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="L9">
         <v>1609</v>
@@ -1700,7 +1731,7 @@
         <v>1</v>
       </c>
       <c r="O9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="P9">
         <v>40</v>
@@ -1712,7 +1743,7 @@
         <v>1</v>
       </c>
       <c r="S9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="T9">
         <v>40</v>
@@ -1724,10 +1755,10 @@
         <v>1</v>
       </c>
       <c r="W9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="X9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Y9">
         <v>40</v>
@@ -1739,10 +1770,10 @@
         <v>1</v>
       </c>
       <c r="AB9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="AD9">
         <v>40</v>
@@ -1754,10 +1785,10 @@
         <v>1</v>
       </c>
       <c r="AG9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AH9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="AI9">
         <v>40</v>
@@ -1786,8 +1817,11 @@
       <c r="AQ9">
         <v>97.513983840894966</v>
       </c>
+      <c r="AR9">
+        <v>1.9264941141965239</v>
+      </c>
     </row>
-    <row r="10" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>8</v>
       </c>
@@ -1795,7 +1829,7 @@
         <v>57</v>
       </c>
       <c r="C10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D10">
         <v>3357</v>
@@ -1807,19 +1841,19 @@
         <v>1</v>
       </c>
       <c r="G10">
-        <v>3325.0942811978439</v>
+        <v>3338.5792246608871</v>
       </c>
       <c r="H10">
-        <v>375.71286905536999</v>
+        <v>216.9179260871245</v>
       </c>
       <c r="I10">
         <v>100</v>
       </c>
       <c r="J10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="L10">
         <v>3357</v>
@@ -1831,7 +1865,7 @@
         <v>1</v>
       </c>
       <c r="O10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="P10">
         <v>3357</v>
@@ -1843,7 +1877,7 @@
         <v>1</v>
       </c>
       <c r="S10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="T10">
         <v>3357</v>
@@ -1855,10 +1889,10 @@
         <v>1</v>
       </c>
       <c r="W10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="X10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Y10">
         <v>3357</v>
@@ -1870,10 +1904,10 @@
         <v>1</v>
       </c>
       <c r="AB10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="AD10">
         <v>3357</v>
@@ -1885,10 +1919,10 @@
         <v>1</v>
       </c>
       <c r="AG10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AH10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="AI10">
         <v>3357</v>
@@ -1917,8 +1951,11 @@
       <c r="AQ10">
         <v>0</v>
       </c>
+      <c r="AR10">
+        <v>0.54872729636917883</v>
+      </c>
     </row>
-    <row r="11" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>9</v>
       </c>
@@ -1926,7 +1963,7 @@
         <v>78</v>
       </c>
       <c r="C11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D11">
         <v>-4028</v>
@@ -1938,19 +1975,19 @@
         <v>1</v>
       </c>
       <c r="G11">
-        <v>-4029.4891397464248</v>
+        <v>-4029.0529808128308</v>
       </c>
       <c r="H11">
-        <v>273.57539912817651</v>
+        <v>193.44701988934989</v>
       </c>
       <c r="I11">
         <v>100</v>
       </c>
       <c r="J11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L11">
         <v>-4028</v>
@@ -1962,7 +1999,7 @@
         <v>1</v>
       </c>
       <c r="O11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="P11">
         <v>-4028</v>
@@ -1974,7 +2011,7 @@
         <v>1</v>
       </c>
       <c r="S11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="T11">
         <v>-4028</v>
@@ -1986,10 +2023,10 @@
         <v>1</v>
       </c>
       <c r="W11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="X11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="Y11">
         <v>-4028</v>
@@ -2001,10 +2038,10 @@
         <v>1</v>
       </c>
       <c r="AB11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="AD11">
         <v>-4028</v>
@@ -2016,10 +2053,10 @@
         <v>1</v>
       </c>
       <c r="AG11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AH11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="AI11">
         <v>-4028</v>
@@ -2047,6 +2084,9 @@
       </c>
       <c r="AQ11">
         <v>0</v>
+      </c>
+      <c r="AR11">
+        <v>2.614152961348722E-2</v>
       </c>
     </row>
   </sheetData>
@@ -2056,47 +2096,50 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B2">
         <v>10</v>
@@ -2123,10 +2166,13 @@
         <v>874.4</v>
       </c>
       <c r="J2">
-        <v>1206.2921981811519</v>
+        <v>1267.504115819931</v>
       </c>
       <c r="K2">
         <v>0.93311758360302055</v>
+      </c>
+      <c r="L2">
+        <v>0.46541559584978531</v>
       </c>
     </row>
   </sheetData>

</xml_diff>